<commit_message>
Excel: Tare Houses çay ve kahve kalemlerindeki yanlış fotoğraf dosyası adları kaldırıldı
İkisi de başka ürünün/otelin fotoğrafını gösteriyordu; Foto Durumu zaten Çekilecek.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XmtctKudQTsHwvjcEf4d9L
</commit_message>
<xml_diff>
--- a/data/HK_Veri_Toplama.xlsx
+++ b/data/HK_Veri_Toplama.xlsx
@@ -10956,9 +10956,7 @@
         <v>526</v>
       </c>
       <c r="E84" s="5"/>
-      <c r="F84" s="7" t="s">
-        <v>527</v>
-      </c>
+      <c r="F84" s="7"/>
       <c r="G84" s="5" t="s">
         <v>281</v>
       </c>
@@ -10981,9 +10979,7 @@
         <v>526</v>
       </c>
       <c r="E85" s="5"/>
-      <c r="F85" s="7" t="s">
-        <v>530</v>
-      </c>
+      <c r="F85" s="7"/>
       <c r="G85" s="5" t="s">
         <v>281</v>
       </c>

</xml_diff>

<commit_message>
X1 ve X2 şablonları oda videolarıyla düzeltildi
- X2: banyo, ikram tepsisi, servis çekmecesi videodan doğrulandı; yemek alanı ve TV adımı eklendi (20 adım)
- X1: banyo havlu askıları, cam paravanlı duş, klima ve çöp kovası doğrulandı; genel oda iki kare (yatak odası + oturma)
- Fotoğrafı olmayan adımlara videodan referans kare
- Excel, fixture ve karar 22 güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XmtctKudQTsHwvjcEf4d9L
</commit_message>
<xml_diff>
--- a/data/HK_Veri_Toplama.xlsx
+++ b/data/HK_Veri_Toplama.xlsx
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
@@ -1466,7 +1466,9 @@
           <t>X2</t>
         </is>
       </c>
-      <c r="C26" s="5" t="n"/>
+      <c r="C26" s="5" t="n">
+        <v>9</v>
+      </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
           <t>İkram tepsisi</t>
@@ -1485,11 +1487,7 @@
       <c r="G26" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı (3 kişilikte 3 olabilir)</t>
-        </is>
-      </c>
+      <c r="H26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1502,7 +1500,9 @@
           <t>X2</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n"/>
+      <c r="C27" s="5" t="n">
+        <v>9</v>
+      </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
           <t>İkram tepsisi</t>
@@ -1521,11 +1521,7 @@
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı (3 kişilikte 3 olabilir)</t>
-        </is>
-      </c>
+      <c r="H27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1538,7 +1534,9 @@
           <t>X2</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n"/>
+      <c r="C28" s="5" t="n">
+        <v>9</v>
+      </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
           <t>İkram tepsisi</t>
@@ -1557,11 +1555,7 @@
       <c r="G28" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı (3 kişilikte 3 olabilir)</t>
-        </is>
-      </c>
+      <c r="H28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1574,7 +1568,9 @@
           <t>X2</t>
         </is>
       </c>
-      <c r="C29" s="5" t="n"/>
+      <c r="C29" s="5" t="n">
+        <v>9</v>
+      </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
           <t>İkram tepsisi</t>
@@ -1593,11 +1589,7 @@
       <c r="G29" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı (3 kişilikte 3 olabilir)</t>
-        </is>
-      </c>
+      <c r="H29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1610,7 +1602,9 @@
           <t>X2</t>
         </is>
       </c>
-      <c r="C30" s="5" t="n"/>
+      <c r="C30" s="5" t="n">
+        <v>9</v>
+      </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
           <t>İkram tepsisi</t>
@@ -1629,11 +1623,7 @@
       <c r="G30" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı (3 kişilikte 3 olabilir)</t>
-        </is>
-      </c>
+      <c r="H30" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -7819,7 +7809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L258"/>
+  <dimension ref="A1:L259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20034,7 +20024,7 @@
       </c>
       <c r="E220" s="5" t="inlineStr">
         <is>
-          <t>Kapıyı açık bırak, odanın içinden kapıya doğru çek: kapı kolu/kilit, TV ve duvar dipleri görünsün.</t>
+          <t>Yatak odasında, yatağın yanından giriş kapısına doğru çek: şifreli kilitli kapı, TV ve duvar dipleri görünsün.</t>
         </is>
       </c>
       <c r="F220" s="5" t="inlineStr">
@@ -20104,7 +20094,8 @@
 Batarya parlak, su lekesi yok
 Sıvı sabun dolu
 LED ayna lekesiz, ışığı yanıyor
-Tezgah kuru</t>
+Tezgah kuru
+Havlu askısında 1 banyo havlusu, halkalarda el havlusu asılı</t>
         </is>
       </c>
       <c r="G221" s="5" t="inlineStr">
@@ -20280,13 +20271,14 @@
       </c>
       <c r="E224" s="5" t="inlineStr">
         <is>
-          <t>Duşu tam karşıdan çek: tepe duşu, el duşu, 3 dispenser ve köşe sepeti görünsün. Cam varsa ikinci açıyı ışığa karşı al.</t>
+          <t>Kapısız, cam paravanlı duşu karşıdan çek: tepe duşu, el duşu, 3 dispenser, köşe sepeti ve lineer gider görünsün. İkinci açıda camı ışığa karşı al.</t>
         </is>
       </c>
       <c r="F224" s="5" t="inlineStr">
         <is>
-          <t>Duvar ve zemin kireçsiz, su lekesi yok
-Giderde saç yok
+          <t>Cam paravanda kireç ve su lekesi yok
+Duvar ve zemin temiz
+Lineer giderde saç yok
 3 dispenser dolu (şampuan, saç kremi, duş jeli)
 El duşu askıda
 Köşe sepeti boş</t>
@@ -20596,7 +20588,8 @@
 Cam sehpa lekesiz
 Halı düz, saçaklar düzgün
 Perde ve tül düzgün
-Aplikler ve lambader yanıyor</t>
+Aplikler ve lambader yanıyor
+Balkon kapısı kapalı ve kilitli, camı lekesiz</t>
         </is>
       </c>
       <c r="G229" s="5" t="inlineStr">
@@ -21194,13 +21187,13 @@
       </c>
       <c r="E239" s="5" t="inlineStr">
         <is>
-          <t>Kapı tarafından tüm odayı tek geniş karede çek. Tüm ışıklar açık.</t>
+          <t>1. kare: yatak odası, giriş kapısının yanından. 2. kare: oturma + mutfak bölümü, iç kapıdan balkona doğru. Tüm ışıklar açık.</t>
         </is>
       </c>
       <c r="F239" s="5" t="inlineStr">
         <is>
-          <t>Klima çalışıyor
-Oda çöp kovası boş
+          <t>Klima çalışıyor (oturma bölümü)
+Masa altındaki çöp kovası boş
 Zemin temiz
 Duvarda iz/sıyrık yok
 Tüm aydınlatma yanıyor</t>
@@ -21227,7 +21220,7 @@
         </is>
       </c>
       <c r="K239" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -21256,7 +21249,7 @@
       </c>
       <c r="E240" s="5" t="inlineStr">
         <is>
-          <t>Kapıdan içeri girince yatağa doğru çek: konsol masa, yatak ve kapı kasası aynı karede.</t>
+          <t>Giriş kapısının içinden odaya doğru çek: yatak, konsol masa, kanepe ve pencere tarafı aynı karede.</t>
         </is>
       </c>
       <c r="F240" s="5" t="inlineStr">
@@ -21326,7 +21319,8 @@
 Batarya parlak, su lekesi yok
 Sıvı sabun dolu
 LED ayna lekesiz, ışığı yanıyor
-Tezgah kuru</t>
+Tezgah kuru
+Havlu askısında 2 banyo havlusu asılı</t>
         </is>
       </c>
       <c r="G241" s="5" t="inlineStr">
@@ -21384,10 +21378,10 @@
       </c>
       <c r="F242" s="5" t="inlineStr">
         <is>
-          <t>3 banyo + 3 el havlusu katlı ve lekesiz (3 kişilik)
-3 çift terlik poşetinde
+          <t>2 banyo + 2 el havlusu katlı (askıdakiler hariç)
+2 çift terlik poşetinde
 Yedek tuvalet kağıdı var
-Saç kurutma makinesi yerinde</t>
+Saç kurutma makinesi yerinde, kablosu toplanmış</t>
         </is>
       </c>
       <c r="G242" s="5" t="inlineStr">
@@ -21502,17 +21496,18 @@
       </c>
       <c r="E244" s="5" t="inlineStr">
         <is>
-          <t>Duşu tam karşıdan çek: tepe duşu, el duşu, 3 dispenser ve köşe sepeti görünsün. Cam varsa ikinci açıyı ışığa karşı al.</t>
+          <t>Kapısız, cam paravanlı duşu karşıdan çek: tepe duşu, el duşu, 3 dispenser, köşe sepeti ve lineer gider görünsün. İkinci açıda camı ışığa karşı al.</t>
         </is>
       </c>
       <c r="F244" s="5" t="inlineStr">
         <is>
-          <t>Duvar ve zemin kireçsiz, su lekesi yok
-Giderde saç yok
+          <t>Cam paravanda kireç ve su lekesi yok
+Duvar ve zemin temiz
+Lineer giderde saç yok
 3 dispenser dolu (şampuan, saç kremi, duş jeli)
 El duşu askıda
 Köşe sepeti boş
-Banyo cam kapısı ve siyah çerçevesi lekesiz</t>
+Banyonun buzlu cam kapısı lekesiz</t>
         </is>
       </c>
       <c r="G244" s="5" t="inlineStr">
@@ -21743,20 +21738,21 @@
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>İkram ve kumandalar</t>
+          <t>Yemek masası: ikram ve kumandalar</t>
         </is>
       </c>
       <c r="E248" s="5" t="inlineStr">
         <is>
-          <t>İkram tepsisini ve kumandaları üstten tek karede çek; paketler yan yana dizili.</t>
+          <t>Yuvarlak yemek masasının üstünü çek: ikram tepsisi ve iki kumanda aynı karede, paketler yan yana.</t>
         </is>
       </c>
       <c r="F248" s="5" t="inlineStr">
         <is>
-          <t>3 fincan + bambu altlık (3 kişilik; teyit et)
+          <t>2 fincan + bambu altlık ters kapatılmış
 Lokum kasesi dolu
-Türk kahvesi, yeşil çay, Nescafe, kahve kreması, toz şeker tam
-TV ve klima kumandası yerinde</t>
+Türk kahvesi 2, yeşil çay 2, Nescafe 2, kahve kreması 2, toz şeker 2
+TV ve klima kumandası yerinde
+Masa tozsuz</t>
         </is>
       </c>
       <c r="G248" s="5" t="inlineStr">
@@ -21809,7 +21805,7 @@
       </c>
       <c r="E249" s="5" t="inlineStr">
         <is>
-          <t>Yatak tarafından pencereye doğru geniş açıyla çek: kanepe (sofa yatak), cam sehpa, halı, perdeler ve aplikler görünsün.</t>
+          <t>Kanepenin karşısından çek: kanepe, cam sehpa, halı, mutfak nişinin perdesi ve kolon görünsün.</t>
         </is>
       </c>
       <c r="F249" s="5" t="inlineStr">
@@ -21817,7 +21813,7 @@
           <t>Sofa yatak toplanmış, minderler düzgün (3. kişi kullandıysa çarşafı alınmış)
 Cam sehpa lekesiz
 Halı düz, saçaklar düzgün
-Perde ve tül düzgün
+Mutfak nişinin perdesi düzgün
 Aplikler yanıyor
 Dekoratif dallar yerinde</t>
         </is>
@@ -21862,20 +21858,82 @@
       </c>
       <c r="C250" s="5" t="inlineStr">
         <is>
+          <t>Oda</t>
+        </is>
+      </c>
+      <c r="D250" s="5" t="inlineStr">
+        <is>
+          <t>Yemek alanı ve TV</t>
+        </is>
+      </c>
+      <c r="E250" s="5" t="inlineStr">
+        <is>
+          <t>Yatağın ayak ucundan pencereye doğru çek: yuvarlak masa, iki berjer, lambader, perde ve duvardaki TV görünsün.</t>
+        </is>
+      </c>
+      <c r="F250" s="5" t="inlineStr">
+        <is>
+          <t>Yuvarlak masa temiz
+2 berjer düzgün, lekesiz
+Lambader yanıyor
+Perde ve tül düzgün, pencere kapalı
+TV ekranı tozsuz</t>
+        </is>
+      </c>
+      <c r="G250" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H250" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="I250" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J250" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>1</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Masada, berjerlerde kir, leke veya eşya var mı? Perde düzgün mü? TV ekranında toz var mı? (Konaklama kontrolündeysen misafir eşyalarını değerlendirme.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C251" s="5" t="inlineStr">
+        <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D250" s="5" t="inlineStr">
+      <c r="D251" s="5" t="inlineStr">
         <is>
           <t>Mutfak tezgahı</t>
         </is>
       </c>
-      <c r="E250" s="5" t="inlineStr">
-        <is>
-          <t>Mutfağın karşısından çek: ocak, evye, batarya, sünger standı, asma çöp kovası, buzdolabı ve açık raflar tek karede.</t>
-        </is>
-      </c>
-      <c r="F250" s="5" t="inlineStr">
+      <c r="E251" s="5" t="inlineStr">
+        <is>
+          <t>Perdeyi aç, mutfak nişinin karşısından çek: ocak, evye, sünger standı, bulaşıklık, asma çöp kovası, buzdolabı ve üst raflar tek karede; solda banyo kapısı.</t>
+        </is>
+      </c>
+      <c r="F251" s="5" t="inlineStr">
         <is>
           <t>2 gözlü ocak camı temiz
 Evye ve batarya temiz
@@ -21885,60 +21943,60 @@
 Buzdolabı kapağı kapalı ve temiz</t>
         </is>
       </c>
-      <c r="G250" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H250" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="I250" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="J250" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K250" t="n">
-        <v>1</v>
-      </c>
-      <c r="L250" t="inlineStr">
+      <c r="G251" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H251" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="I251" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J251" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>1</v>
+      </c>
+      <c r="L251" t="inlineStr">
         <is>
           <t>Ocakta yanık veya yağ lekesi var mı? Evyede bulaşık var mı? Bulaşıklıkta eşya var mı? Çöp kovası dolu mu? (Konaklama kontrolündeysen misafir eşyalarını değerlendirme.)</t>
         </is>
       </c>
     </row>
-    <row r="251">
-      <c r="A251" s="5" t="inlineStr">
+    <row r="252">
+      <c r="A252" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B251" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="C251" s="5" t="inlineStr">
+      <c r="B252" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C252" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D251" s="5" t="inlineStr">
+      <c r="D252" s="5" t="inlineStr">
         <is>
           <t>Çekmece 1: çatal-bıçak</t>
         </is>
       </c>
-      <c r="E251" s="5" t="inlineStr">
+      <c r="E252" s="5" t="inlineStr">
         <is>
           <t>Çekmeceyi tamamen aç, feneri aç, tam üstten çek. Çatal-bıçaklar üst üste binmesin.</t>
         </is>
       </c>
-      <c r="F251" s="5" t="inlineStr">
+      <c r="F252" s="5" t="inlineStr">
         <is>
           <t>Çatal, kaşık, bıçak ve çay kaşığı tam
 Şarap açacağı yerinde
@@ -21946,178 +22004,178 @@
 Kaşıklık altı kırıntısız</t>
         </is>
       </c>
-      <c r="G251" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H251" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I251" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J251" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K251" t="n">
-        <v>1</v>
-      </c>
-      <c r="L251" t="inlineStr">
+      <c r="G252" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H252" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I252" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J252" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>1</v>
+      </c>
+      <c r="L252" t="inlineStr">
         <is>
           <t>Her bölmedeki yemek kaşığı, çatal, bıçak ve çay kaşığını ayrı say. Setle aynı olmayan parça var mı?</t>
         </is>
       </c>
     </row>
-    <row r="252">
-      <c r="A252" s="5" t="inlineStr">
+    <row r="253">
+      <c r="A253" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B252" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C252" s="5" t="inlineStr">
+      <c r="B253" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C253" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D252" s="5" t="inlineStr">
+      <c r="D253" s="5" t="inlineStr">
         <is>
           <t>Çekmece 2: servis gereçleri</t>
         </is>
       </c>
-      <c r="E252" s="5" t="inlineStr">
+      <c r="E253" s="5" t="inlineStr">
         <is>
           <t>Çekmeceyi tamamen aç, feneri aç, üstten çek.</t>
         </is>
       </c>
-      <c r="F252" s="5" t="inlineStr">
+      <c r="F253" s="5" t="inlineStr">
         <is>
           <t>4 silikon servis gereci (kepçe, delikli kepçe, kaşık, spatula)
 Çekmece içi kırıntısız</t>
         </is>
       </c>
-      <c r="G252" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H252" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I252" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J252" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K252" t="n">
-        <v>1</v>
-      </c>
-      <c r="L252" t="inlineStr">
+      <c r="G253" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H253" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I253" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J253" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>1</v>
+      </c>
+      <c r="L253" t="inlineStr">
         <is>
           <t>Kaç silikon servis gereci var? Hangileri eksik?</t>
         </is>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="5" t="inlineStr">
+    <row r="254">
+      <c r="A254" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B253" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="C253" s="5" t="inlineStr">
+      <c r="B254" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C254" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D253" s="5" t="inlineStr">
+      <c r="D254" s="5" t="inlineStr">
         <is>
           <t>Çekmece 3: bıçak seti</t>
         </is>
       </c>
-      <c r="E253" s="5" t="inlineStr">
+      <c r="E254" s="5" t="inlineStr">
         <is>
           <t>Çekmeceyi tamamen aç; bıçak seti kutusu açık ve kesme tahtası görünsün.</t>
         </is>
       </c>
-      <c r="F253" s="5" t="inlineStr">
+      <c r="F254" s="5" t="inlineStr">
         <is>
           <t>Bıçak seti tam (kutuda)
 Kesme tahtası temiz</t>
         </is>
       </c>
-      <c r="G253" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H253" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I253" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J253" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K253" t="n">
-        <v>1</v>
-      </c>
-      <c r="L253" t="inlineStr">
+      <c r="G254" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H254" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I254" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J254" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>1</v>
+      </c>
+      <c r="L254" t="inlineStr">
         <is>
           <t>Bıçak setinde boş yuva var mı? Kesme tahtasında leke veya küf var mı?</t>
         </is>
       </c>
     </row>
-    <row r="254">
-      <c r="A254" s="5" t="inlineStr">
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B254" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="C254" s="5" t="inlineStr">
+      <c r="B255" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C255" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D254" s="5" t="inlineStr">
+      <c r="D255" s="5" t="inlineStr">
         <is>
           <t>Açık raf: tabak ve kase</t>
         </is>
       </c>
-      <c r="E254" s="5" t="inlineStr">
+      <c r="E255" s="5" t="inlineStr">
         <is>
           <t>Açık raf bölümünü önden çek; tabak ve kase yığınları yandan sayılabilsin.</t>
         </is>
       </c>
-      <c r="F254" s="5" t="inlineStr">
+      <c r="F255" s="5" t="inlineStr">
         <is>
           <t>6 kase (zeytin yeşili)
 4 küçük gri tabak
@@ -22126,60 +22184,60 @@
 Tabaklarda iz veya çatlak yok</t>
         </is>
       </c>
-      <c r="G254" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H254" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I254" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J254" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K254" t="n">
-        <v>1</v>
-      </c>
-      <c r="L254" t="inlineStr">
+      <c r="G255" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H255" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I255" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J255" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>1</v>
+      </c>
+      <c r="L255" t="inlineStr">
         <is>
           <t>Kase, küçük tabak, büyük düz tabak ve gri tabak sayısını yığınlardan ayrı say. Çatlak veya leke var mı?</t>
         </is>
       </c>
     </row>
-    <row r="255">
-      <c r="A255" s="5" t="inlineStr">
+    <row r="256">
+      <c r="A256" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B255" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="C255" s="5" t="inlineStr">
+      <c r="B256" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C256" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D255" s="5" t="inlineStr">
+      <c r="D256" s="5" t="inlineStr">
         <is>
           <t>Üst dolap: kupa, fincan, bardak</t>
         </is>
       </c>
-      <c r="E255" s="5" t="inlineStr">
+      <c r="E256" s="5" t="inlineStr">
         <is>
           <t>Kapağı aç, feneri aç; kupalar, fincan tabakları ve bardaklar yan yana görünsün.</t>
         </is>
       </c>
-      <c r="F255" s="5" t="inlineStr">
+      <c r="F256" s="5" t="inlineStr">
         <is>
           <t>2 kupa + 3 küçük fincan
 Fincan tabakları tam
@@ -22188,60 +22246,60 @@
 Bardaklarda su lekesi yok</t>
         </is>
       </c>
-      <c r="G255" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H255" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I255" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J255" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K255" t="n">
-        <v>1</v>
-      </c>
-      <c r="L255" t="inlineStr">
+      <c r="G256" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H256" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I256" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J256" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>1</v>
+      </c>
+      <c r="L256" t="inlineStr">
         <is>
           <t>Kupa, küçük fincan, fincan tabağı, su bardağı, kısa bardak, kadeh ve küçük kaseyi ayrı say. Bardaklarda leke var mı?</t>
         </is>
       </c>
     </row>
-    <row r="256">
-      <c r="A256" s="5" t="inlineStr">
+    <row r="257">
+      <c r="A257" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B256" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="C256" s="5" t="inlineStr">
+      <c r="B257" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C257" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D256" s="5" t="inlineStr">
+      <c r="D257" s="5" t="inlineStr">
         <is>
           <t>Evye altı: tencere-tava</t>
         </is>
       </c>
-      <c r="E256" s="5" t="inlineStr">
+      <c r="E257" s="5" t="inlineStr">
         <is>
           <t>Kapakları aç, feneri aç; iki rafı da görecek şekilde çek.</t>
         </is>
       </c>
-      <c r="F256" s="5" t="inlineStr">
+      <c r="F257" s="5" t="inlineStr">
         <is>
           <t>Tencere ve tava kapaklarıyla tam
 Tava içi temiz
@@ -22249,60 +22307,60 @@
 Sifonda sızıntı yok</t>
         </is>
       </c>
-      <c r="G256" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H256" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I256" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="J256" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K256" t="n">
-        <v>1</v>
-      </c>
-      <c r="L256" t="inlineStr">
+      <c r="G257" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H257" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I257" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J257" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>1</v>
+      </c>
+      <c r="L257" t="inlineStr">
         <is>
           <t>Kaç tencere ve tava var, kapakları var mı? Tava içinde yağ kalıntısı var mı? Dolap tabanında su var mı?</t>
         </is>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="5" t="inlineStr">
+    <row r="258">
+      <c r="A258" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B257" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="C257" s="5" t="inlineStr">
+      <c r="B258" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
         <is>
           <t>Mutfak</t>
         </is>
       </c>
-      <c r="D257" s="5" t="inlineStr">
+      <c r="D258" s="5" t="inlineStr">
         <is>
           <t>Mini buzdolabı</t>
         </is>
       </c>
-      <c r="E257" s="5" t="inlineStr">
+      <c r="E258" s="5" t="inlineStr">
         <is>
           <t>Kapağı tamamen aç; içi ve kapak rafları görünsün.</t>
         </is>
       </c>
-      <c r="F257" s="5" t="inlineStr">
+      <c r="F258" s="5" t="inlineStr">
         <is>
           <t>Raflar ve kapak rafları temiz
 Misafirden kalan yiyecek/içecek yok
@@ -22310,60 +22368,60 @@
 Kapak rafındaki su şişeleri tam</t>
         </is>
       </c>
-      <c r="G257" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H257" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="I257" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="J257" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K257" t="n">
-        <v>1</v>
-      </c>
-      <c r="L257" t="inlineStr">
+      <c r="G258" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H258" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="I258" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J258" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>1</v>
+      </c>
+      <c r="L258" t="inlineStr">
         <is>
           <t>Buzdolabında misafirden kalan yiyecek/içecek var mı? Raflarda leke veya buzlanma var mı?</t>
         </is>
       </c>
     </row>
-    <row r="258">
-      <c r="A258" s="5" t="inlineStr">
+    <row r="259">
+      <c r="A259" s="5" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B258" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="C258" s="5" t="inlineStr">
+      <c r="B259" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C259" s="5" t="inlineStr">
         <is>
           <t>Oda</t>
         </is>
       </c>
-      <c r="D258" s="5" t="inlineStr">
+      <c r="D259" s="5" t="inlineStr">
         <is>
           <t>Genel oda</t>
         </is>
       </c>
-      <c r="E258" s="5" t="inlineStr">
+      <c r="E259" s="5" t="inlineStr">
         <is>
           <t>Kapı tarafından tüm odayı tek geniş karede çek. Tüm ışıklar açık.</t>
         </is>
       </c>
-      <c r="F258" s="5" t="inlineStr">
+      <c r="F259" s="5" t="inlineStr">
         <is>
           <t>Klima çalışıyor
 Oda çöp kovası boş
@@ -22372,30 +22430,30 @@
 Tüm aydınlatma yanıyor</t>
         </is>
       </c>
-      <c r="G258" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="H258" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="I258" s="5" t="inlineStr">
-        <is>
-          <t>Hayır</t>
-        </is>
-      </c>
-      <c r="J258" s="5" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="K258" t="n">
-        <v>1</v>
-      </c>
-      <c r="L258" t="inlineStr">
+      <c r="G259" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="H259" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="I259" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J259" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="K259" t="n">
+        <v>1</v>
+      </c>
+      <c r="L259" t="inlineStr">
         <is>
           <t>Zeminde kir veya çöp var mı? Açıkta kablo var mı? Duvarda iz var mı? Yanmayan lamba var mı? (Konaklama kontrolündeysen misafir eşyalarını değerlendirme.)</t>
         </is>
@@ -30332,7 +30390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K500"/>
+  <dimension ref="A1:K507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -49966,7 +50024,7 @@
       </c>
       <c r="K414" s="5" t="inlineStr">
         <is>
-          <t>2024 notunda 2 TV yazıyordu; yeni fotoğraflarda yatak karşısında 1 TV var. Odada say.</t>
+          <t>Yatak odasında 1 TV (video); oturma bölümünde TV yok</t>
         </is>
       </c>
     </row>
@@ -50166,7 +50224,7 @@
         </is>
       </c>
       <c r="C419" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D419">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B419)*('Kontrol Adımları'!$B$1:$B$400=C419),0),0)),"")</f>
@@ -50174,7 +50232,7 @@
       </c>
       <c r="E419" s="5" t="inlineStr">
         <is>
-          <t>bath_towel</t>
+          <t>towel_bar</t>
         </is>
       </c>
       <c r="F419">
@@ -50186,7 +50244,7 @@
         <v/>
       </c>
       <c r="H419" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I419" s="7" t="inlineStr">
         <is>
@@ -50212,7 +50270,7 @@
         </is>
       </c>
       <c r="C420" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D420">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B420)*('Kontrol Adımları'!$B$1:$B$400=C420),0),0)),"")</f>
@@ -50220,7 +50278,7 @@
       </c>
       <c r="E420" s="5" t="inlineStr">
         <is>
-          <t>hand_towel</t>
+          <t>towel_ring</t>
         </is>
       </c>
       <c r="F420">
@@ -50244,7 +50302,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K420" s="5" t="n"/>
+      <c r="K420" s="5" t="inlineStr">
+        <is>
+          <t>Lavabo yanında + duşta</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="5" t="inlineStr">
@@ -50266,7 +50328,7 @@
       </c>
       <c r="E421" s="5" t="inlineStr">
         <is>
-          <t>slippers</t>
+          <t>bath_towel</t>
         </is>
       </c>
       <c r="F421">
@@ -50312,7 +50374,7 @@
       </c>
       <c r="E422" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_spare</t>
+          <t>hand_towel</t>
         </is>
       </c>
       <c r="F422">
@@ -50324,7 +50386,7 @@
         <v/>
       </c>
       <c r="H422" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I422" s="7" t="inlineStr">
         <is>
@@ -50358,7 +50420,7 @@
       </c>
       <c r="E423" s="5" t="inlineStr">
         <is>
-          <t>hair_dryer</t>
+          <t>slippers</t>
         </is>
       </c>
       <c r="F423">
@@ -50370,7 +50432,7 @@
         <v/>
       </c>
       <c r="H423" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I423" s="7" t="inlineStr">
         <is>
@@ -50404,7 +50466,7 @@
       </c>
       <c r="E424" s="5" t="inlineStr">
         <is>
-          <t>vanity_unit</t>
+          <t>toilet_paper_spare</t>
         </is>
       </c>
       <c r="F424">
@@ -50442,7 +50504,7 @@
         </is>
       </c>
       <c r="C425" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D425">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B425)*('Kontrol Adımları'!$B$1:$B$400=C425),0),0)),"")</f>
@@ -50450,7 +50512,7 @@
       </c>
       <c r="E425" s="5" t="inlineStr">
         <is>
-          <t>wc</t>
+          <t>hair_dryer</t>
         </is>
       </c>
       <c r="F425">
@@ -50488,7 +50550,7 @@
         </is>
       </c>
       <c r="C426" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D426">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B426)*('Kontrol Adımları'!$B$1:$B$400=C426),0),0)),"")</f>
@@ -50496,7 +50558,7 @@
       </c>
       <c r="E426" s="5" t="inlineStr">
         <is>
-          <t>flush_plate</t>
+          <t>vanity_unit</t>
         </is>
       </c>
       <c r="F426">
@@ -50542,7 +50604,7 @@
       </c>
       <c r="E427" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper</t>
+          <t>wc</t>
         </is>
       </c>
       <c r="F427">
@@ -50588,7 +50650,7 @@
       </c>
       <c r="E428" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_holder</t>
+          <t>flush_plate</t>
         </is>
       </c>
       <c r="F428">
@@ -50634,7 +50696,7 @@
       </c>
       <c r="E429" s="5" t="inlineStr">
         <is>
-          <t>toilet_brush</t>
+          <t>toilet_paper</t>
         </is>
       </c>
       <c r="F429">
@@ -50680,7 +50742,7 @@
       </c>
       <c r="E430" s="5" t="inlineStr">
         <is>
-          <t>bath_bin</t>
+          <t>toilet_paper_holder</t>
         </is>
       </c>
       <c r="F430">
@@ -50718,7 +50780,7 @@
         </is>
       </c>
       <c r="C431" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D431">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B431)*('Kontrol Adımları'!$B$1:$B$400=C431),0),0)),"")</f>
@@ -50726,7 +50788,7 @@
       </c>
       <c r="E431" s="5" t="inlineStr">
         <is>
-          <t>shower_set</t>
+          <t>toilet_brush</t>
         </is>
       </c>
       <c r="F431">
@@ -50764,7 +50826,7 @@
         </is>
       </c>
       <c r="C432" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D432">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B432)*('Kontrol Adımları'!$B$1:$B$400=C432),0),0)),"")</f>
@@ -50772,7 +50834,7 @@
       </c>
       <c r="E432" s="5" t="inlineStr">
         <is>
-          <t>dispenser</t>
+          <t>bath_bin</t>
         </is>
       </c>
       <c r="F432">
@@ -50784,7 +50846,7 @@
         <v/>
       </c>
       <c r="H432" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I432" s="7" t="inlineStr">
         <is>
@@ -50818,7 +50880,7 @@
       </c>
       <c r="E433" s="5" t="inlineStr">
         <is>
-          <t>shower_basket</t>
+          <t>shower_set</t>
         </is>
       </c>
       <c r="F433">
@@ -50856,7 +50918,7 @@
         </is>
       </c>
       <c r="C434" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D434">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B434)*('Kontrol Adımları'!$B$1:$B$400=C434),0),0)),"")</f>
@@ -50864,7 +50926,7 @@
       </c>
       <c r="E434" s="5" t="inlineStr">
         <is>
-          <t>bed</t>
+          <t>dispenser</t>
         </is>
       </c>
       <c r="F434">
@@ -50876,7 +50938,7 @@
         <v/>
       </c>
       <c r="H434" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I434" s="7" t="inlineStr">
         <is>
@@ -50902,7 +50964,7 @@
         </is>
       </c>
       <c r="C435" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D435">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B435)*('Kontrol Adımları'!$B$1:$B$400=C435),0),0)),"")</f>
@@ -50910,7 +50972,7 @@
       </c>
       <c r="E435" s="5" t="inlineStr">
         <is>
-          <t>pillow</t>
+          <t>shower_basket</t>
         </is>
       </c>
       <c r="F435">
@@ -50922,7 +50984,7 @@
         <v/>
       </c>
       <c r="H435" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I435" s="7" t="inlineStr">
         <is>
@@ -50948,7 +51010,7 @@
         </is>
       </c>
       <c r="C436" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D436">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B436)*('Kontrol Adımları'!$B$1:$B$400=C436),0),0)),"")</f>
@@ -50956,7 +51018,7 @@
       </c>
       <c r="E436" s="5" t="inlineStr">
         <is>
-          <t>nightstand</t>
+          <t>bed</t>
         </is>
       </c>
       <c r="F436">
@@ -50968,7 +51030,7 @@
         <v/>
       </c>
       <c r="H436" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I436" s="7" t="inlineStr">
         <is>
@@ -50994,7 +51056,7 @@
         </is>
       </c>
       <c r="C437" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D437">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B437)*('Kontrol Adımları'!$B$1:$B$400=C437),0),0)),"")</f>
@@ -51002,7 +51064,7 @@
       </c>
       <c r="E437" s="5" t="inlineStr">
         <is>
-          <t>bedside_wall_lamp</t>
+          <t>pillow</t>
         </is>
       </c>
       <c r="F437">
@@ -51014,7 +51076,7 @@
         <v/>
       </c>
       <c r="H437" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I437" s="7" t="inlineStr">
         <is>
@@ -51040,7 +51102,7 @@
         </is>
       </c>
       <c r="C438" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D438">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B438)*('Kontrol Adımları'!$B$1:$B$400=C438),0),0)),"")</f>
@@ -51048,7 +51110,7 @@
       </c>
       <c r="E438" s="5" t="inlineStr">
         <is>
-          <t>wardrobe</t>
+          <t>nightstand</t>
         </is>
       </c>
       <c r="F438">
@@ -51060,7 +51122,7 @@
         <v/>
       </c>
       <c r="H438" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I438" s="7" t="inlineStr">
         <is>
@@ -51086,7 +51148,7 @@
         </is>
       </c>
       <c r="C439" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D439">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B439)*('Kontrol Adımları'!$B$1:$B$400=C439),0),0)),"")</f>
@@ -51094,7 +51156,7 @@
       </c>
       <c r="E439" s="5" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>bedside_wall_lamp</t>
         </is>
       </c>
       <c r="F439">
@@ -51106,7 +51168,7 @@
         <v/>
       </c>
       <c r="H439" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I439" s="7" t="inlineStr">
         <is>
@@ -51118,11 +51180,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K439" s="5" t="inlineStr">
-        <is>
-          <t>5 siyah ahşap + 1 şeffaf</t>
-        </is>
-      </c>
+      <c r="K439" s="5" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="5" t="inlineStr">
@@ -51144,7 +51202,7 @@
       </c>
       <c r="E440" s="5" t="inlineStr">
         <is>
-          <t>spare_blanket</t>
+          <t>wardrobe</t>
         </is>
       </c>
       <c r="F440">
@@ -51182,7 +51240,7 @@
         </is>
       </c>
       <c r="C441" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D441">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B441)*('Kontrol Adımları'!$B$1:$B$400=C441),0),0)),"")</f>
@@ -51190,7 +51248,7 @@
       </c>
       <c r="E441" s="5" t="inlineStr">
         <is>
-          <t>desk_with_chair</t>
+          <t>hanger</t>
         </is>
       </c>
       <c r="F441">
@@ -51202,7 +51260,7 @@
         <v/>
       </c>
       <c r="H441" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I441" s="7" t="inlineStr">
         <is>
@@ -51214,7 +51272,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K441" s="5" t="n"/>
+      <c r="K441" s="5" t="inlineStr">
+        <is>
+          <t>5 siyah ahşap + 1 şeffaf</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="5" t="inlineStr">
@@ -51228,7 +51290,7 @@
         </is>
       </c>
       <c r="C442" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D442">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B442)*('Kontrol Adımları'!$B$1:$B$400=C442),0),0)),"")</f>
@@ -51236,7 +51298,7 @@
       </c>
       <c r="E442" s="5" t="inlineStr">
         <is>
-          <t>amenity_tray</t>
+          <t>spare_blanket</t>
         </is>
       </c>
       <c r="F442">
@@ -51282,7 +51344,7 @@
       </c>
       <c r="E443" s="5" t="inlineStr">
         <is>
-          <t>remote</t>
+          <t>desk_with_chair</t>
         </is>
       </c>
       <c r="F443">
@@ -51294,7 +51356,7 @@
         <v/>
       </c>
       <c r="H443" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I443" s="7" t="inlineStr">
         <is>
@@ -51320,7 +51382,7 @@
         </is>
       </c>
       <c r="C444" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D444">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B444)*('Kontrol Adımları'!$B$1:$B$400=C444),0),0)),"")</f>
@@ -51328,7 +51390,7 @@
       </c>
       <c r="E444" s="5" t="inlineStr">
         <is>
-          <t>sofa_gray</t>
+          <t>amenity_tray</t>
         </is>
       </c>
       <c r="F444">
@@ -51366,7 +51428,7 @@
         </is>
       </c>
       <c r="C445" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D445">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B445)*('Kontrol Adımları'!$B$1:$B$400=C445),0),0)),"")</f>
@@ -51374,7 +51436,7 @@
       </c>
       <c r="E445" s="5" t="inlineStr">
         <is>
-          <t>coffee_table_glass</t>
+          <t>remote</t>
         </is>
       </c>
       <c r="F445">
@@ -51386,7 +51448,7 @@
         <v/>
       </c>
       <c r="H445" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I445" s="7" t="inlineStr">
         <is>
@@ -51420,7 +51482,7 @@
       </c>
       <c r="E446" s="5" t="inlineStr">
         <is>
-          <t>floor_lamp</t>
+          <t>sofa_gray</t>
         </is>
       </c>
       <c r="F446">
@@ -51466,7 +51528,7 @@
       </c>
       <c r="E447" s="5" t="inlineStr">
         <is>
-          <t>rug_striped</t>
+          <t>coffee_table_glass</t>
         </is>
       </c>
       <c r="F447">
@@ -51512,7 +51574,7 @@
       </c>
       <c r="E448" s="5" t="inlineStr">
         <is>
-          <t>round_wall_lamp</t>
+          <t>floor_lamp</t>
         </is>
       </c>
       <c r="F448">
@@ -51524,7 +51586,7 @@
         <v/>
       </c>
       <c r="H448" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I448" s="7" t="inlineStr">
         <is>
@@ -51558,7 +51620,7 @@
       </c>
       <c r="E449" s="5" t="inlineStr">
         <is>
-          <t>wall_art</t>
+          <t>rug_striped</t>
         </is>
       </c>
       <c r="F449">
@@ -51570,7 +51632,7 @@
         <v/>
       </c>
       <c r="H449" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I449" s="7" t="inlineStr">
         <is>
@@ -51582,11 +51644,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K449" s="5" t="inlineStr">
-        <is>
-          <t>Yatak üstü + oturma alanı</t>
-        </is>
-      </c>
+      <c r="K449" s="5" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="5" t="inlineStr">
@@ -51600,7 +51658,7 @@
         </is>
       </c>
       <c r="C450" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D450">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B450)*('Kontrol Adımları'!$B$1:$B$400=C450),0),0)),"")</f>
@@ -51608,7 +51666,7 @@
       </c>
       <c r="E450" s="5" t="inlineStr">
         <is>
-          <t>cooktop</t>
+          <t>round_wall_lamp</t>
         </is>
       </c>
       <c r="F450">
@@ -51620,7 +51678,7 @@
         <v/>
       </c>
       <c r="H450" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I450" s="7" t="inlineStr">
         <is>
@@ -51646,7 +51704,7 @@
         </is>
       </c>
       <c r="C451" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D451">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B451)*('Kontrol Adımları'!$B$1:$B$400=C451),0),0)),"")</f>
@@ -51654,7 +51712,7 @@
       </c>
       <c r="E451" s="5" t="inlineStr">
         <is>
-          <t>hanging_bin</t>
+          <t>wall_art</t>
         </is>
       </c>
       <c r="F451">
@@ -51666,7 +51724,7 @@
         <v/>
       </c>
       <c r="H451" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I451" s="7" t="inlineStr">
         <is>
@@ -51678,7 +51736,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K451" s="5" t="n"/>
+      <c r="K451" s="5" t="inlineStr">
+        <is>
+          <t>Yatak üstü + oturma alanı</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="5" t="inlineStr">
@@ -51700,7 +51762,7 @@
       </c>
       <c r="E452" s="5" t="inlineStr">
         <is>
-          <t>mini_fridge</t>
+          <t>cooktop</t>
         </is>
       </c>
       <c r="F452">
@@ -51746,7 +51808,7 @@
       </c>
       <c r="E453" s="5" t="inlineStr">
         <is>
-          <t>range_hood</t>
+          <t>hanging_bin</t>
         </is>
       </c>
       <c r="F453">
@@ -51762,7 +51824,7 @@
       </c>
       <c r="I453" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J453" s="5" t="inlineStr">
@@ -51770,11 +51832,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K453" s="5" t="inlineStr">
-        <is>
-          <t>Üst dolap altında görünüyor</t>
-        </is>
-      </c>
+      <c r="K453" s="5" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="5" t="inlineStr">
@@ -51788,7 +51846,7 @@
         </is>
       </c>
       <c r="C454" s="5" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D454">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B454)*('Kontrol Adımları'!$B$1:$B$400=C454),0),0)),"")</f>
@@ -51796,7 +51854,7 @@
       </c>
       <c r="E454" s="5" t="inlineStr">
         <is>
-          <t>kettle</t>
+          <t>mini_fridge</t>
         </is>
       </c>
       <c r="F454">
@@ -51834,7 +51892,7 @@
         </is>
       </c>
       <c r="C455" s="5" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D455">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B455)*('Kontrol Adımları'!$B$1:$B$400=C455),0),0)),"")</f>
@@ -51842,7 +51900,7 @@
       </c>
       <c r="E455" s="5" t="inlineStr">
         <is>
-          <t>paper_towel</t>
+          <t>range_hood</t>
         </is>
       </c>
       <c r="F455">
@@ -51868,7 +51926,7 @@
       </c>
       <c r="K455" s="5" t="inlineStr">
         <is>
-          <t>X2 ile aynı varsayıldı</t>
+          <t>Üst dolap altında görünüyor</t>
         </is>
       </c>
     </row>
@@ -51884,7 +51942,7 @@
         </is>
       </c>
       <c r="C456" s="5" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D456">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B456)*('Kontrol Adımları'!$B$1:$B$400=C456),0),0)),"")</f>
@@ -51892,7 +51950,7 @@
       </c>
       <c r="E456" s="5" t="inlineStr">
         <is>
-          <t>air_conditioner</t>
+          <t>kettle</t>
         </is>
       </c>
       <c r="F456">
@@ -51908,7 +51966,7 @@
       </c>
       <c r="I456" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J456" s="5" t="inlineStr">
@@ -51916,11 +51974,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K456" s="5" t="inlineStr">
-        <is>
-          <t>Fotoğraflarda görünmüyor; yerini teyit et</t>
-        </is>
-      </c>
+      <c r="K456" s="5" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="5" t="inlineStr">
@@ -51934,7 +51988,7 @@
         </is>
       </c>
       <c r="C457" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D457">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B457)*('Kontrol Adımları'!$B$1:$B$400=C457),0),0)),"")</f>
@@ -51942,7 +51996,7 @@
       </c>
       <c r="E457" s="5" t="inlineStr">
         <is>
-          <t>room_bin</t>
+          <t>paper_towel</t>
         </is>
       </c>
       <c r="F457">
@@ -51968,7 +52022,7 @@
       </c>
       <c r="K457" s="5" t="inlineStr">
         <is>
-          <t>Fotoğraflarda görünmüyor</t>
+          <t>X2 ile aynı varsayıldı</t>
         </is>
       </c>
     </row>
@@ -51980,11 +52034,11 @@
       </c>
       <c r="B458" s="5" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="C458" s="5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D458">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B458)*('Kontrol Adımları'!$B$1:$B$400=C458),0),0)),"")</f>
@@ -51992,7 +52046,7 @@
       </c>
       <c r="E458" s="5" t="inlineStr">
         <is>
-          <t>desk_with_chair</t>
+          <t>air_conditioner</t>
         </is>
       </c>
       <c r="F458">
@@ -52016,7 +52070,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K458" s="5" t="n"/>
+      <c r="K458" s="5" t="inlineStr">
+        <is>
+          <t>Oturma bölümünde, banyo kapısının üstünde (video)</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="5" t="inlineStr">
@@ -52026,11 +52084,11 @@
       </c>
       <c r="B459" s="5" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="C459" s="5" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D459">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B459)*('Kontrol Adımları'!$B$1:$B$400=C459),0),0)),"")</f>
@@ -52038,7 +52096,7 @@
       </c>
       <c r="E459" s="5" t="inlineStr">
         <is>
-          <t>vessel_sink</t>
+          <t>room_bin</t>
         </is>
       </c>
       <c r="F459">
@@ -52054,7 +52112,7 @@
       </c>
       <c r="I459" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J459" s="5" t="inlineStr">
@@ -52064,7 +52122,7 @@
       </c>
       <c r="K459" s="5" t="inlineStr">
         <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
+          <t>Video</t>
         </is>
       </c>
     </row>
@@ -52080,7 +52138,7 @@
         </is>
       </c>
       <c r="C460" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D460">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B460)*('Kontrol Adımları'!$B$1:$B$400=C460),0),0)),"")</f>
@@ -52088,7 +52146,7 @@
       </c>
       <c r="E460" s="5" t="inlineStr">
         <is>
-          <t>basin_faucet</t>
+          <t>desk_with_chair</t>
         </is>
       </c>
       <c r="F460">
@@ -52104,7 +52162,7 @@
       </c>
       <c r="I460" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J460" s="5" t="inlineStr">
@@ -52112,11 +52170,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K460" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K460" s="5" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="5" t="inlineStr">
@@ -52138,7 +52192,7 @@
       </c>
       <c r="E461" s="5" t="inlineStr">
         <is>
-          <t>led_mirror</t>
+          <t>vessel_sink</t>
         </is>
       </c>
       <c r="F461">
@@ -52154,7 +52208,7 @@
       </c>
       <c r="I461" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J461" s="5" t="inlineStr">
@@ -52162,11 +52216,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K461" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K461" s="5" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="5" t="inlineStr">
@@ -52188,7 +52238,7 @@
       </c>
       <c r="E462" s="5" t="inlineStr">
         <is>
-          <t>liquid_soap</t>
+          <t>basin_faucet</t>
         </is>
       </c>
       <c r="F462">
@@ -52204,7 +52254,7 @@
       </c>
       <c r="I462" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J462" s="5" t="inlineStr">
@@ -52212,11 +52262,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K462" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K462" s="5" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="5" t="inlineStr">
@@ -52230,7 +52276,7 @@
         </is>
       </c>
       <c r="C463" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D463">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B463)*('Kontrol Adımları'!$B$1:$B$400=C463),0),0)),"")</f>
@@ -52238,7 +52284,7 @@
       </c>
       <c r="E463" s="5" t="inlineStr">
         <is>
-          <t>bath_towel</t>
+          <t>led_mirror</t>
         </is>
       </c>
       <c r="F463">
@@ -52250,11 +52296,11 @@
         <v/>
       </c>
       <c r="H463" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I463" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J463" s="5" t="inlineStr">
@@ -52262,11 +52308,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K463" s="5" t="inlineStr">
-        <is>
-          <t>3 kişilik oda; teyit et</t>
-        </is>
-      </c>
+      <c r="K463" s="5" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="5" t="inlineStr">
@@ -52280,7 +52322,7 @@
         </is>
       </c>
       <c r="C464" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D464">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B464)*('Kontrol Adımları'!$B$1:$B$400=C464),0),0)),"")</f>
@@ -52288,7 +52330,7 @@
       </c>
       <c r="E464" s="5" t="inlineStr">
         <is>
-          <t>hand_towel</t>
+          <t>liquid_soap</t>
         </is>
       </c>
       <c r="F464">
@@ -52300,11 +52342,11 @@
         <v/>
       </c>
       <c r="H464" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I464" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J464" s="5" t="inlineStr">
@@ -52312,11 +52354,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K464" s="5" t="inlineStr">
-        <is>
-          <t>3 kişilik oda; teyit et</t>
-        </is>
-      </c>
+      <c r="K464" s="5" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="5" t="inlineStr">
@@ -52330,7 +52368,7 @@
         </is>
       </c>
       <c r="C465" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D465">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B465)*('Kontrol Adımları'!$B$1:$B$400=C465),0),0)),"")</f>
@@ -52338,7 +52376,7 @@
       </c>
       <c r="E465" s="5" t="inlineStr">
         <is>
-          <t>slippers</t>
+          <t>towel_bar</t>
         </is>
       </c>
       <c r="F465">
@@ -52350,11 +52388,11 @@
         <v/>
       </c>
       <c r="H465" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I465" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J465" s="5" t="inlineStr">
@@ -52362,11 +52400,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K465" s="5" t="inlineStr">
-        <is>
-          <t>3 kişilik oda; teyit et</t>
-        </is>
-      </c>
+      <c r="K465" s="5" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="5" t="inlineStr">
@@ -52388,7 +52422,7 @@
       </c>
       <c r="E466" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_spare</t>
+          <t>bath_towel</t>
         </is>
       </c>
       <c r="F466">
@@ -52400,11 +52434,11 @@
         <v/>
       </c>
       <c r="H466" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I466" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J466" s="5" t="inlineStr">
@@ -52412,11 +52446,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K466" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K466" s="5" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="5" t="inlineStr">
@@ -52438,7 +52468,7 @@
       </c>
       <c r="E467" s="5" t="inlineStr">
         <is>
-          <t>hair_dryer</t>
+          <t>hand_towel</t>
         </is>
       </c>
       <c r="F467">
@@ -52450,11 +52480,11 @@
         <v/>
       </c>
       <c r="H467" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I467" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J467" s="5" t="inlineStr">
@@ -52462,11 +52492,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K467" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K467" s="5" t="n"/>
     </row>
     <row r="468" ht="26.4" customHeight="1">
       <c r="A468" s="5" t="inlineStr">
@@ -52488,7 +52514,7 @@
       </c>
       <c r="E468" s="5" t="inlineStr">
         <is>
-          <t>vanity_unit</t>
+          <t>slippers</t>
         </is>
       </c>
       <c r="F468">
@@ -52500,11 +52526,11 @@
         <v/>
       </c>
       <c r="H468" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I468" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J468" s="5" t="inlineStr">
@@ -52512,11 +52538,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K468" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K468" s="5" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="5" t="inlineStr">
@@ -52530,7 +52552,7 @@
         </is>
       </c>
       <c r="C469" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D469">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B469)*('Kontrol Adımları'!$B$1:$B$400=C469),0),0)),"")</f>
@@ -52538,7 +52560,7 @@
       </c>
       <c r="E469" s="5" t="inlineStr">
         <is>
-          <t>wc</t>
+          <t>toilet_paper_spare</t>
         </is>
       </c>
       <c r="F469">
@@ -52554,7 +52576,7 @@
       </c>
       <c r="I469" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J469" s="5" t="inlineStr">
@@ -52562,11 +52584,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K469" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K469" s="5" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="5" t="inlineStr">
@@ -52580,7 +52598,7 @@
         </is>
       </c>
       <c r="C470" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D470">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B470)*('Kontrol Adımları'!$B$1:$B$400=C470),0),0)),"")</f>
@@ -52588,7 +52606,7 @@
       </c>
       <c r="E470" s="5" t="inlineStr">
         <is>
-          <t>flush_plate</t>
+          <t>hair_dryer</t>
         </is>
       </c>
       <c r="F470">
@@ -52604,7 +52622,7 @@
       </c>
       <c r="I470" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J470" s="5" t="inlineStr">
@@ -52612,11 +52630,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K470" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K470" s="5" t="n"/>
     </row>
     <row r="471" ht="26.4" customHeight="1">
       <c r="A471" s="5" t="inlineStr">
@@ -52630,7 +52644,7 @@
         </is>
       </c>
       <c r="C471" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D471">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B471)*('Kontrol Adımları'!$B$1:$B$400=C471),0),0)),"")</f>
@@ -52638,7 +52652,7 @@
       </c>
       <c r="E471" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper</t>
+          <t>vanity_unit</t>
         </is>
       </c>
       <c r="F471">
@@ -52654,7 +52668,7 @@
       </c>
       <c r="I471" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J471" s="5" t="inlineStr">
@@ -52662,11 +52676,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K471" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K471" s="5" t="n"/>
     </row>
     <row r="472" ht="26.4" customHeight="1">
       <c r="A472" s="5" t="inlineStr">
@@ -52688,7 +52698,7 @@
       </c>
       <c r="E472" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_holder</t>
+          <t>wc</t>
         </is>
       </c>
       <c r="F472">
@@ -52704,7 +52714,7 @@
       </c>
       <c r="I472" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J472" s="5" t="inlineStr">
@@ -52712,11 +52722,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K472" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K472" s="5" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="5" t="inlineStr">
@@ -52738,7 +52744,7 @@
       </c>
       <c r="E473" s="5" t="inlineStr">
         <is>
-          <t>toilet_brush</t>
+          <t>flush_plate</t>
         </is>
       </c>
       <c r="F473">
@@ -52754,7 +52760,7 @@
       </c>
       <c r="I473" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J473" s="5" t="inlineStr">
@@ -52762,11 +52768,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K473" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K473" s="5" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="5" t="inlineStr">
@@ -52788,7 +52790,7 @@
       </c>
       <c r="E474" s="5" t="inlineStr">
         <is>
-          <t>bath_bin</t>
+          <t>toilet_paper</t>
         </is>
       </c>
       <c r="F474">
@@ -52804,7 +52806,7 @@
       </c>
       <c r="I474" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J474" s="5" t="inlineStr">
@@ -52812,11 +52814,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K474" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K474" s="5" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="5" t="inlineStr">
@@ -52830,7 +52828,7 @@
         </is>
       </c>
       <c r="C475" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D475">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B475)*('Kontrol Adımları'!$B$1:$B$400=C475),0),0)),"")</f>
@@ -52838,7 +52836,7 @@
       </c>
       <c r="E475" s="5" t="inlineStr">
         <is>
-          <t>shower_set</t>
+          <t>toilet_paper_holder</t>
         </is>
       </c>
       <c r="F475">
@@ -52854,7 +52852,7 @@
       </c>
       <c r="I475" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J475" s="5" t="inlineStr">
@@ -52862,11 +52860,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K475" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K475" s="5" t="n"/>
     </row>
     <row r="476" ht="26.4" customHeight="1">
       <c r="A476" s="5" t="inlineStr">
@@ -52880,7 +52874,7 @@
         </is>
       </c>
       <c r="C476" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D476">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B476)*('Kontrol Adımları'!$B$1:$B$400=C476),0),0)),"")</f>
@@ -52888,7 +52882,7 @@
       </c>
       <c r="E476" s="5" t="inlineStr">
         <is>
-          <t>dispenser</t>
+          <t>toilet_brush</t>
         </is>
       </c>
       <c r="F476">
@@ -52900,11 +52894,11 @@
         <v/>
       </c>
       <c r="H476" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I476" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J476" s="5" t="inlineStr">
@@ -52912,11 +52906,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K476" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K476" s="5" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="5" t="inlineStr">
@@ -52930,7 +52920,7 @@
         </is>
       </c>
       <c r="C477" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D477">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B477)*('Kontrol Adımları'!$B$1:$B$400=C477),0),0)),"")</f>
@@ -52938,7 +52928,7 @@
       </c>
       <c r="E477" s="5" t="inlineStr">
         <is>
-          <t>shower_basket</t>
+          <t>bath_bin</t>
         </is>
       </c>
       <c r="F477">
@@ -52954,7 +52944,7 @@
       </c>
       <c r="I477" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J477" s="5" t="inlineStr">
@@ -52962,11 +52952,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K477" s="5" t="inlineStr">
-        <is>
-          <t>X2 banyo fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K477" s="5" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="5" t="inlineStr">
@@ -52980,7 +52966,7 @@
         </is>
       </c>
       <c r="C478" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D478">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B478)*('Kontrol Adımları'!$B$1:$B$400=C478),0),0)),"")</f>
@@ -52988,7 +52974,7 @@
       </c>
       <c r="E478" s="5" t="inlineStr">
         <is>
-          <t>bed</t>
+          <t>shower_set</t>
         </is>
       </c>
       <c r="F478">
@@ -53026,7 +53012,7 @@
         </is>
       </c>
       <c r="C479" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D479">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B479)*('Kontrol Adımları'!$B$1:$B$400=C479),0),0)),"")</f>
@@ -53034,7 +53020,7 @@
       </c>
       <c r="E479" s="5" t="inlineStr">
         <is>
-          <t>pillow</t>
+          <t>dispenser</t>
         </is>
       </c>
       <c r="F479">
@@ -53046,7 +53032,7 @@
         <v/>
       </c>
       <c r="H479" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I479" s="7" t="inlineStr">
         <is>
@@ -53072,7 +53058,7 @@
         </is>
       </c>
       <c r="C480" s="5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D480">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B480)*('Kontrol Adımları'!$B$1:$B$400=C480),0),0)),"")</f>
@@ -53080,7 +53066,7 @@
       </c>
       <c r="E480" s="5" t="inlineStr">
         <is>
-          <t>nightstand</t>
+          <t>shower_basket</t>
         </is>
       </c>
       <c r="F480">
@@ -53092,7 +53078,7 @@
         <v/>
       </c>
       <c r="H480" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I480" s="7" t="inlineStr">
         <is>
@@ -53118,7 +53104,7 @@
         </is>
       </c>
       <c r="C481" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D481">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B481)*('Kontrol Adımları'!$B$1:$B$400=C481),0),0)),"")</f>
@@ -53126,7 +53112,7 @@
       </c>
       <c r="E481" s="5" t="inlineStr">
         <is>
-          <t>bedside_wall_lamp</t>
+          <t>bed</t>
         </is>
       </c>
       <c r="F481">
@@ -53138,7 +53124,7 @@
         <v/>
       </c>
       <c r="H481" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I481" s="7" t="inlineStr">
         <is>
@@ -53164,7 +53150,7 @@
         </is>
       </c>
       <c r="C482" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D482">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B482)*('Kontrol Adımları'!$B$1:$B$400=C482),0),0)),"")</f>
@@ -53172,7 +53158,7 @@
       </c>
       <c r="E482" s="5" t="inlineStr">
         <is>
-          <t>wardrobe</t>
+          <t>pillow</t>
         </is>
       </c>
       <c r="F482">
@@ -53184,7 +53170,7 @@
         <v/>
       </c>
       <c r="H482" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I482" s="7" t="inlineStr">
         <is>
@@ -53210,7 +53196,7 @@
         </is>
       </c>
       <c r="C483" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D483">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B483)*('Kontrol Adımları'!$B$1:$B$400=C483),0),0)),"")</f>
@@ -53218,7 +53204,7 @@
       </c>
       <c r="E483" s="5" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>nightstand</t>
         </is>
       </c>
       <c r="F483">
@@ -53230,11 +53216,11 @@
         <v/>
       </c>
       <c r="H483" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I483" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J483" s="5" t="inlineStr">
@@ -53242,11 +53228,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K483" s="5" t="inlineStr">
-        <is>
-          <t>Askılar sola toplanmış; fotoğrafta 4-5 görünüyor</t>
-        </is>
-      </c>
+      <c r="K483" s="5" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="5" t="inlineStr">
@@ -53260,7 +53242,7 @@
         </is>
       </c>
       <c r="C484" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D484">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B484)*('Kontrol Adımları'!$B$1:$B$400=C484),0),0)),"")</f>
@@ -53268,7 +53250,7 @@
       </c>
       <c r="E484" s="5" t="inlineStr">
         <is>
-          <t>spare_blanket</t>
+          <t>bedside_wall_lamp</t>
         </is>
       </c>
       <c r="F484">
@@ -53280,7 +53262,7 @@
         <v/>
       </c>
       <c r="H484" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I484" s="7" t="inlineStr">
         <is>
@@ -53306,7 +53288,7 @@
         </is>
       </c>
       <c r="C485" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D485">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B485)*('Kontrol Adımları'!$B$1:$B$400=C485),0),0)),"")</f>
@@ -53314,7 +53296,7 @@
       </c>
       <c r="E485" s="5" t="inlineStr">
         <is>
-          <t>amenity_tray</t>
+          <t>wardrobe</t>
         </is>
       </c>
       <c r="F485">
@@ -53330,7 +53312,7 @@
       </c>
       <c r="I485" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J485" s="5" t="inlineStr">
@@ -53338,11 +53320,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K485" s="5" t="inlineStr">
-        <is>
-          <t>X2 ikram fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K485" s="5" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="5" t="inlineStr">
@@ -53356,7 +53334,7 @@
         </is>
       </c>
       <c r="C486" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D486">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B486)*('Kontrol Adımları'!$B$1:$B$400=C486),0),0)),"")</f>
@@ -53364,7 +53342,7 @@
       </c>
       <c r="E486" s="5" t="inlineStr">
         <is>
-          <t>remote</t>
+          <t>hanger</t>
         </is>
       </c>
       <c r="F486">
@@ -53376,7 +53354,7 @@
         <v/>
       </c>
       <c r="H486" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I486" s="7" t="inlineStr">
         <is>
@@ -53390,7 +53368,7 @@
       </c>
       <c r="K486" s="5" t="inlineStr">
         <is>
-          <t>X1 ile aynı varsayıldı</t>
+          <t>Askılar sola toplanmış; fotoğrafta 4-5 görünüyor</t>
         </is>
       </c>
     </row>
@@ -53406,7 +53384,7 @@
         </is>
       </c>
       <c r="C487" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D487">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B487)*('Kontrol Adımları'!$B$1:$B$400=C487),0),0)),"")</f>
@@ -53414,7 +53392,7 @@
       </c>
       <c r="E487" s="5" t="inlineStr">
         <is>
-          <t>sofa_gray</t>
+          <t>spare_blanket</t>
         </is>
       </c>
       <c r="F487">
@@ -53452,7 +53430,7 @@
         </is>
       </c>
       <c r="C488" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D488">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B488)*('Kontrol Adımları'!$B$1:$B$400=C488),0),0)),"")</f>
@@ -53460,7 +53438,7 @@
       </c>
       <c r="E488" s="5" t="inlineStr">
         <is>
-          <t>coffee_table_glass</t>
+          <t>amenity_tray</t>
         </is>
       </c>
       <c r="F488">
@@ -53498,7 +53476,7 @@
         </is>
       </c>
       <c r="C489" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D489">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B489)*('Kontrol Adımları'!$B$1:$B$400=C489),0),0)),"")</f>
@@ -53506,7 +53484,7 @@
       </c>
       <c r="E489" s="5" t="inlineStr">
         <is>
-          <t>rug_striped</t>
+          <t>remote</t>
         </is>
       </c>
       <c r="F489">
@@ -53518,7 +53496,7 @@
         <v/>
       </c>
       <c r="H489" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I489" s="7" t="inlineStr">
         <is>
@@ -53552,7 +53530,7 @@
       </c>
       <c r="E490" s="5" t="inlineStr">
         <is>
-          <t>round_wall_lamp</t>
+          <t>sofa_gray</t>
         </is>
       </c>
       <c r="F490">
@@ -53564,7 +53542,7 @@
         <v/>
       </c>
       <c r="H490" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I490" s="7" t="inlineStr">
         <is>
@@ -53598,7 +53576,7 @@
       </c>
       <c r="E491" s="5" t="inlineStr">
         <is>
-          <t>decor_branches</t>
+          <t>coffee_table_glass</t>
         </is>
       </c>
       <c r="F491">
@@ -53644,7 +53622,7 @@
       </c>
       <c r="E492" s="5" t="inlineStr">
         <is>
-          <t>wall_art</t>
+          <t>rug_striped</t>
         </is>
       </c>
       <c r="F492">
@@ -53668,11 +53646,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K492" s="5" t="inlineStr">
-        <is>
-          <t>Yatak üstünde</t>
-        </is>
-      </c>
+      <c r="K492" s="5" t="n"/>
     </row>
     <row r="493" ht="26.4" customHeight="1">
       <c r="A493" s="5" t="inlineStr">
@@ -53686,7 +53660,7 @@
         </is>
       </c>
       <c r="C493" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D493">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B493)*('Kontrol Adımları'!$B$1:$B$400=C493),0),0)),"")</f>
@@ -53694,7 +53668,7 @@
       </c>
       <c r="E493" s="5" t="inlineStr">
         <is>
-          <t>cooktop</t>
+          <t>round_wall_lamp</t>
         </is>
       </c>
       <c r="F493">
@@ -53706,7 +53680,7 @@
         <v/>
       </c>
       <c r="H493" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I493" s="7" t="inlineStr">
         <is>
@@ -53732,7 +53706,7 @@
         </is>
       </c>
       <c r="C494" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D494">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B494)*('Kontrol Adımları'!$B$1:$B$400=C494),0),0)),"")</f>
@@ -53740,7 +53714,7 @@
       </c>
       <c r="E494" s="5" t="inlineStr">
         <is>
-          <t>hanging_bin</t>
+          <t>decor_branches</t>
         </is>
       </c>
       <c r="F494">
@@ -53778,7 +53752,7 @@
         </is>
       </c>
       <c r="C495" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D495">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B495)*('Kontrol Adımları'!$B$1:$B$400=C495),0),0)),"")</f>
@@ -53786,7 +53760,7 @@
       </c>
       <c r="E495" s="5" t="inlineStr">
         <is>
-          <t>mini_fridge</t>
+          <t>wall_art</t>
         </is>
       </c>
       <c r="F495">
@@ -53810,7 +53784,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K495" s="5" t="n"/>
+      <c r="K495" s="5" t="inlineStr">
+        <is>
+          <t>Yatak üstünde</t>
+        </is>
+      </c>
     </row>
     <row r="496">
       <c r="A496" s="5" t="inlineStr">
@@ -53832,7 +53810,7 @@
       </c>
       <c r="E496" s="5" t="inlineStr">
         <is>
-          <t>range_hood</t>
+          <t>round_table</t>
         </is>
       </c>
       <c r="F496">
@@ -53878,7 +53856,7 @@
       </c>
       <c r="E497" s="5" t="inlineStr">
         <is>
-          <t>kettle</t>
+          <t>armchair</t>
         </is>
       </c>
       <c r="F497">
@@ -53890,7 +53868,7 @@
         <v/>
       </c>
       <c r="H497" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I497" s="7" t="inlineStr">
         <is>
@@ -53916,7 +53894,7 @@
         </is>
       </c>
       <c r="C498" s="5" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D498">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B498)*('Kontrol Adımları'!$B$1:$B$400=C498),0),0)),"")</f>
@@ -53924,7 +53902,7 @@
       </c>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>paper_towel</t>
+          <t>floor_lamp</t>
         </is>
       </c>
       <c r="F498">
@@ -53962,7 +53940,7 @@
         </is>
       </c>
       <c r="C499" s="5" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D499">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B499)*('Kontrol Adımları'!$B$1:$B$400=C499),0),0)),"")</f>
@@ -53970,7 +53948,7 @@
       </c>
       <c r="E499" s="5" t="inlineStr">
         <is>
-          <t>air_conditioner</t>
+          <t>tv</t>
         </is>
       </c>
       <c r="F499">
@@ -53986,7 +53964,7 @@
       </c>
       <c r="I499" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J499" s="5" t="inlineStr">
@@ -53994,11 +53972,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K499" s="5" t="inlineStr">
-        <is>
-          <t>Fotoğraflarda görünmüyor</t>
-        </is>
-      </c>
+      <c r="K499" s="5" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="5" t="inlineStr">
@@ -54012,7 +53986,7 @@
         </is>
       </c>
       <c r="C500" s="5" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D500">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B500)*('Kontrol Adımları'!$B$1:$B$400=C500),0),0)),"")</f>
@@ -54020,7 +53994,7 @@
       </c>
       <c r="E500" s="5" t="inlineStr">
         <is>
-          <t>room_bin</t>
+          <t>cooktop</t>
         </is>
       </c>
       <c r="F500">
@@ -54036,7 +54010,7 @@
       </c>
       <c r="I500" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J500" s="5" t="inlineStr">
@@ -54044,7 +54018,333 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K500" s="5" t="inlineStr">
+      <c r="K500" s="5" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B501" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C501" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D501">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B501)*('Kontrol Adımları'!$B$1:$B$400=C501),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E501" s="5" t="inlineStr">
+        <is>
+          <t>hanging_bin</t>
+        </is>
+      </c>
+      <c r="F501">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A501)*('Kalem Kataloğu'!$B$1:$B$1000=E501),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G501">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A501)*('Kalem Kataloğu'!$B$1:$B$1000=E501),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H501" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I501" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J501" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K501" s="5" t="n"/>
+    </row>
+    <row r="502">
+      <c r="A502" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B502" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C502" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D502">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B502)*('Kontrol Adımları'!$B$1:$B$400=C502),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E502" s="5" t="inlineStr">
+        <is>
+          <t>mini_fridge</t>
+        </is>
+      </c>
+      <c r="F502">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A502)*('Kalem Kataloğu'!$B$1:$B$1000=E502),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G502">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A502)*('Kalem Kataloğu'!$B$1:$B$1000=E502),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H502" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I502" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J502" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K502" s="5" t="n"/>
+    </row>
+    <row r="503">
+      <c r="A503" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B503" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C503" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D503">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B503)*('Kontrol Adımları'!$B$1:$B$400=C503),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E503" s="5" t="inlineStr">
+        <is>
+          <t>range_hood</t>
+        </is>
+      </c>
+      <c r="F503">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A503)*('Kalem Kataloğu'!$B$1:$B$1000=E503),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G503">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A503)*('Kalem Kataloğu'!$B$1:$B$1000=E503),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H503" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I503" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J503" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K503" s="5" t="n"/>
+    </row>
+    <row r="504">
+      <c r="A504" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B504" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C504" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D504">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B504)*('Kontrol Adımları'!$B$1:$B$400=C504),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E504" s="5" t="inlineStr">
+        <is>
+          <t>kettle</t>
+        </is>
+      </c>
+      <c r="F504">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A504)*('Kalem Kataloğu'!$B$1:$B$1000=E504),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G504">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A504)*('Kalem Kataloğu'!$B$1:$B$1000=E504),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H504" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I504" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J504" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K504" s="5" t="n"/>
+    </row>
+    <row r="505">
+      <c r="A505" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B505" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C505" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D505">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B505)*('Kontrol Adımları'!$B$1:$B$400=C505),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E505" s="5" t="inlineStr">
+        <is>
+          <t>paper_towel</t>
+        </is>
+      </c>
+      <c r="F505">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A505)*('Kalem Kataloğu'!$B$1:$B$1000=E505),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G505">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A505)*('Kalem Kataloğu'!$B$1:$B$1000=E505),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H505" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I505" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J505" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K505" s="5" t="n"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B506" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C506" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D506">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B506)*('Kontrol Adımları'!$B$1:$B$400=C506),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E506" s="5" t="inlineStr">
+        <is>
+          <t>air_conditioner</t>
+        </is>
+      </c>
+      <c r="F506">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A506)*('Kalem Kataloğu'!$B$1:$B$1000=E506),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G506">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A506)*('Kalem Kataloğu'!$B$1:$B$1000=E506),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H506" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I506" s="7" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J506" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K506" s="5" t="inlineStr">
+        <is>
+          <t>Fotoğraflarda görünmüyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B507" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C507" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D507">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B507)*('Kontrol Adımları'!$B$1:$B$400=C507),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E507" s="5" t="inlineStr">
+        <is>
+          <t>room_bin</t>
+        </is>
+      </c>
+      <c r="F507">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A507)*('Kalem Kataloğu'!$B$1:$B$1000=E507),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G507">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A507)*('Kalem Kataloğu'!$B$1:$B$1000=E507),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H507" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I507" s="7" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J507" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K507" s="5" t="inlineStr">
         <is>
           <t>Kanepe yanında siyah kova görünüyor</t>
         </is>
@@ -59373,7 +59673,7 @@
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
@@ -59381,11 +59681,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K112" s="5" t="inlineStr">
-        <is>
-          <t>X1 ile aynı varsayıldı; 3 kişilikte 3 olabilir</t>
-        </is>
-      </c>
+      <c r="K112" s="5" t="n"/>
     </row>
     <row r="113" ht="26.4" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
@@ -59423,7 +59719,7 @@
       </c>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr">
@@ -59431,11 +59727,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K113" s="5" t="inlineStr">
-        <is>
-          <t>X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K113" s="5" t="n"/>
     </row>
     <row r="114" ht="26.4" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
@@ -59449,7 +59741,7 @@
         </is>
       </c>
       <c r="C114" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D114">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B114)*('Kontrol Adımları'!$B$1:$B$400=C114),0),0)),"")</f>
@@ -59495,7 +59787,7 @@
         </is>
       </c>
       <c r="C115" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D115">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B115)*('Kontrol Adımları'!$B$1:$B$400=C115),0),0)),"")</f>
@@ -59541,7 +59833,7 @@
         </is>
       </c>
       <c r="C116" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D116">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B116)*('Kontrol Adımları'!$B$1:$B$400=C116),0),0)),"")</f>
@@ -59587,7 +59879,7 @@
         </is>
       </c>
       <c r="C117" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D117">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B117)*('Kontrol Adımları'!$B$1:$B$400=C117),0),0)),"")</f>
@@ -59633,7 +59925,7 @@
         </is>
       </c>
       <c r="C118" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D118">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B118)*('Kontrol Adımları'!$B$1:$B$400=C118),0),0)),"")</f>
@@ -59679,7 +59971,7 @@
         </is>
       </c>
       <c r="C119" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D119">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B119)*('Kontrol Adımları'!$B$1:$B$400=C119),0),0)),"")</f>
@@ -59729,7 +60021,7 @@
         </is>
       </c>
       <c r="C120" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D120">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B120)*('Kontrol Adımları'!$B$1:$B$400=C120),0),0)),"")</f>
@@ -59779,7 +60071,7 @@
         </is>
       </c>
       <c r="C121" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D121">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B121)*('Kontrol Adımları'!$B$1:$B$400=C121),0),0)),"")</f>
@@ -59829,7 +60121,7 @@
         </is>
       </c>
       <c r="C122" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D122">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B122)*('Kontrol Adımları'!$B$1:$B$400=C122),0),0)),"")</f>
@@ -59879,7 +60171,7 @@
         </is>
       </c>
       <c r="C123" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D123">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B123)*('Kontrol Adımları'!$B$1:$B$400=C123),0),0)),"")</f>
@@ -59925,7 +60217,7 @@
         </is>
       </c>
       <c r="C124" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D124">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B124)*('Kontrol Adımları'!$B$1:$B$400=C124),0),0)),"")</f>
@@ -59949,7 +60241,7 @@
       </c>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J124" s="5" t="inlineStr">
@@ -59957,11 +60249,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K124" s="5" t="inlineStr">
-        <is>
-          <t>X2 fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K124" s="5" t="n"/>
     </row>
     <row r="125" ht="26.4" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
@@ -59975,7 +60263,7 @@
         </is>
       </c>
       <c r="C125" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D125">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B125)*('Kontrol Adımları'!$B$1:$B$400=C125),0),0)),"")</f>
@@ -59999,7 +60287,7 @@
       </c>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr">
@@ -60007,11 +60295,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K125" s="5" t="inlineStr">
-        <is>
-          <t>X2 fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K125" s="5" t="n"/>
     </row>
     <row r="126" ht="26.4" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
@@ -60025,7 +60309,7 @@
         </is>
       </c>
       <c r="C126" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D126">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B126)*('Kontrol Adımları'!$B$1:$B$400=C126),0),0)),"")</f>
@@ -60049,7 +60333,7 @@
       </c>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J126" s="5" t="inlineStr">
@@ -60057,11 +60341,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K126" s="5" t="inlineStr">
-        <is>
-          <t>X2 fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K126" s="5" t="n"/>
     </row>
     <row r="127" ht="26.4" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
@@ -60075,7 +60355,7 @@
         </is>
       </c>
       <c r="C127" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D127">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B127)*('Kontrol Adımları'!$B$1:$B$400=C127),0),0)),"")</f>
@@ -60099,7 +60379,7 @@
       </c>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J127" s="5" t="inlineStr">
@@ -60107,11 +60387,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K127" s="5" t="inlineStr">
-        <is>
-          <t>X2 fotoğrafı yok; X1 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K127" s="5" t="n"/>
     </row>
     <row r="128" ht="26.4" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
@@ -60125,7 +60401,7 @@
         </is>
       </c>
       <c r="C128" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D128">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B128)*('Kontrol Adımları'!$B$1:$B$400=C128),0),0)),"")</f>
@@ -60171,7 +60447,7 @@
         </is>
       </c>
       <c r="C129" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D129">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B129)*('Kontrol Adımları'!$B$1:$B$400=C129),0),0)),"")</f>
@@ -60221,7 +60497,7 @@
         </is>
       </c>
       <c r="C130" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D130">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B130)*('Kontrol Adımları'!$B$1:$B$400=C130),0),0)),"")</f>
@@ -60271,7 +60547,7 @@
         </is>
       </c>
       <c r="C131" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D131">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B131)*('Kontrol Adımları'!$B$1:$B$400=C131),0),0)),"")</f>
@@ -60317,7 +60593,7 @@
         </is>
       </c>
       <c r="C132" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D132">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B132)*('Kontrol Adımları'!$B$1:$B$400=C132),0),0)),"")</f>
@@ -60367,7 +60643,7 @@
         </is>
       </c>
       <c r="C133" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D133">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B133)*('Kontrol Adımları'!$B$1:$B$400=C133),0),0)),"")</f>
@@ -60413,7 +60689,7 @@
         </is>
       </c>
       <c r="C134" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D134">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B134)*('Kontrol Adımları'!$B$1:$B$400=C134),0),0)),"")</f>
@@ -60463,7 +60739,7 @@
         </is>
       </c>
       <c r="C135" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D135">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B135)*('Kontrol Adımları'!$B$1:$B$400=C135),0),0)),"")</f>
@@ -60513,7 +60789,7 @@
         </is>
       </c>
       <c r="C136" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D136">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B136)*('Kontrol Adımları'!$B$1:$B$400=C136),0),0)),"")</f>
@@ -60563,7 +60839,7 @@
         </is>
       </c>
       <c r="C137" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D137">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B137)*('Kontrol Adımları'!$B$1:$B$400=C137),0),0)),"")</f>
@@ -60613,7 +60889,7 @@
         </is>
       </c>
       <c r="C138" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D138">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B138)*('Kontrol Adımları'!$B$1:$B$400=C138),0),0)),"")</f>
@@ -60663,7 +60939,7 @@
         </is>
       </c>
       <c r="C139" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D139">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B139)*('Kontrol Adımları'!$B$1:$B$400=C139),0),0)),"")</f>
@@ -60713,7 +60989,7 @@
         </is>
       </c>
       <c r="C140" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D140">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B140)*('Kontrol Adımları'!$B$1:$B$400=C140),0),0)),"")</f>
@@ -60763,7 +61039,7 @@
         </is>
       </c>
       <c r="C141" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D141">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B141)*('Kontrol Adımları'!$B$1:$B$400=C141),0),0)),"")</f>
@@ -60813,7 +61089,7 @@
         </is>
       </c>
       <c r="C142" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D142">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B142)*('Kontrol Adımları'!$B$1:$B$400=C142),0),0)),"")</f>
@@ -60859,7 +61135,7 @@
         </is>
       </c>
       <c r="C143" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D143">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B143)*('Kontrol Adımları'!$B$1:$B$400=C143),0),0)),"")</f>
@@ -60905,7 +61181,7 @@
         </is>
       </c>
       <c r="C144" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D144">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B144)*('Kontrol Adımları'!$B$1:$B$400=C144),0),0)),"")</f>
@@ -60951,7 +61227,7 @@
         </is>
       </c>
       <c r="C145" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D145">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B145)*('Kontrol Adımları'!$B$1:$B$400=C145),0),0)),"")</f>

</xml_diff>

<commit_message>
X1/X2: aydınlatma kalemleri (tavan armatürü, odadaki LED ayna, duman dedektörü), X2 aplik sayısı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XmtctKudQTsHwvjcEf4d9L
</commit_message>
<xml_diff>
--- a/data/HK_Veri_Toplama.xlsx
+++ b/data/HK_Veri_Toplama.xlsx
@@ -20404,7 +20404,8 @@
 Çekmeceler boş
 Başucu aplikleri yanıyor
 Priz ve anahtarlar sağlam
-Yatak kenarı ve altı temiz</t>
+Yatak kenarı ve altı temiz
+Yatak odasındaki LED ayna lekesiz, ışığı yanıyor</t>
         </is>
       </c>
       <c r="G226" s="5" t="inlineStr">
@@ -22427,7 +22428,8 @@
 Oda çöp kovası boş
 Zemin temiz
 Duvarda iz/sıyrık yok
-Tüm aydınlatma yanıyor</t>
+Tüm aydınlatma yanıyor
+Duman dedektörünün ışığı yanıp sönüyor</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
@@ -22498,7 +22500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I207"/>
+  <dimension ref="A1:I209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -30345,6 +30347,70 @@
         </is>
       </c>
       <c r="H207" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>ceiling_light</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>Tavan armatürü (plafonyer)</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>Demirbaş</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>Yuvarlak tavan armatürü, açık ampullü</t>
+        </is>
+      </c>
+      <c r="H208" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>led_mirror_room</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>Yuvarlak LED ayna (oda)</t>
+        </is>
+      </c>
+      <c r="D209" s="5" t="inlineStr">
+        <is>
+          <t>Demirbaş</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>Yatak odası duvarında, arkadan aydınlatmalı</t>
+        </is>
+      </c>
+      <c r="H209" s="5" t="inlineStr">
         <is>
           <t>Drive foto (20.10.2026)</t>
         </is>
@@ -30390,7 +30456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K507"/>
+  <dimension ref="A1:K510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -51194,7 +51260,7 @@
         </is>
       </c>
       <c r="C440" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D440">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B440)*('Kontrol Adımları'!$B$1:$B$400=C440),0),0)),"")</f>
@@ -51202,7 +51268,7 @@
       </c>
       <c r="E440" s="5" t="inlineStr">
         <is>
-          <t>wardrobe</t>
+          <t>led_mirror_room</t>
         </is>
       </c>
       <c r="F440">
@@ -51226,7 +51292,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K440" s="5" t="n"/>
+      <c r="K440" s="5" t="inlineStr">
+        <is>
+          <t>Yatak odası doğu duvarı (video)</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="5" t="inlineStr">
@@ -51248,7 +51318,7 @@
       </c>
       <c r="E441" s="5" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>wardrobe</t>
         </is>
       </c>
       <c r="F441">
@@ -51260,7 +51330,7 @@
         <v/>
       </c>
       <c r="H441" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I441" s="7" t="inlineStr">
         <is>
@@ -51272,11 +51342,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K441" s="5" t="inlineStr">
-        <is>
-          <t>5 siyah ahşap + 1 şeffaf</t>
-        </is>
-      </c>
+      <c r="K441" s="5" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="5" t="inlineStr">
@@ -51298,7 +51364,7 @@
       </c>
       <c r="E442" s="5" t="inlineStr">
         <is>
-          <t>spare_blanket</t>
+          <t>hanger</t>
         </is>
       </c>
       <c r="F442">
@@ -51310,7 +51376,7 @@
         <v/>
       </c>
       <c r="H442" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I442" s="7" t="inlineStr">
         <is>
@@ -51322,7 +51388,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K442" s="5" t="n"/>
+      <c r="K442" s="5" t="inlineStr">
+        <is>
+          <t>5 siyah ahşap + 1 şeffaf</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="5" t="inlineStr">
@@ -51336,7 +51406,7 @@
         </is>
       </c>
       <c r="C443" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D443">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B443)*('Kontrol Adımları'!$B$1:$B$400=C443),0),0)),"")</f>
@@ -51344,7 +51414,7 @@
       </c>
       <c r="E443" s="5" t="inlineStr">
         <is>
-          <t>desk_with_chair</t>
+          <t>spare_blanket</t>
         </is>
       </c>
       <c r="F443">
@@ -51390,7 +51460,7 @@
       </c>
       <c r="E444" s="5" t="inlineStr">
         <is>
-          <t>amenity_tray</t>
+          <t>desk_with_chair</t>
         </is>
       </c>
       <c r="F444">
@@ -51436,7 +51506,7 @@
       </c>
       <c r="E445" s="5" t="inlineStr">
         <is>
-          <t>remote</t>
+          <t>amenity_tray</t>
         </is>
       </c>
       <c r="F445">
@@ -51448,7 +51518,7 @@
         <v/>
       </c>
       <c r="H445" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I445" s="7" t="inlineStr">
         <is>
@@ -51474,7 +51544,7 @@
         </is>
       </c>
       <c r="C446" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D446">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B446)*('Kontrol Adımları'!$B$1:$B$400=C446),0),0)),"")</f>
@@ -51482,7 +51552,7 @@
       </c>
       <c r="E446" s="5" t="inlineStr">
         <is>
-          <t>sofa_gray</t>
+          <t>remote</t>
         </is>
       </c>
       <c r="F446">
@@ -51494,7 +51564,7 @@
         <v/>
       </c>
       <c r="H446" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I446" s="7" t="inlineStr">
         <is>
@@ -51528,7 +51598,7 @@
       </c>
       <c r="E447" s="5" t="inlineStr">
         <is>
-          <t>coffee_table_glass</t>
+          <t>sofa_gray</t>
         </is>
       </c>
       <c r="F447">
@@ -51574,7 +51644,7 @@
       </c>
       <c r="E448" s="5" t="inlineStr">
         <is>
-          <t>floor_lamp</t>
+          <t>coffee_table_glass</t>
         </is>
       </c>
       <c r="F448">
@@ -51620,7 +51690,7 @@
       </c>
       <c r="E449" s="5" t="inlineStr">
         <is>
-          <t>rug_striped</t>
+          <t>floor_lamp</t>
         </is>
       </c>
       <c r="F449">
@@ -51666,7 +51736,7 @@
       </c>
       <c r="E450" s="5" t="inlineStr">
         <is>
-          <t>round_wall_lamp</t>
+          <t>rug_striped</t>
         </is>
       </c>
       <c r="F450">
@@ -51678,7 +51748,7 @@
         <v/>
       </c>
       <c r="H450" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I450" s="7" t="inlineStr">
         <is>
@@ -51712,7 +51782,7 @@
       </c>
       <c r="E451" s="5" t="inlineStr">
         <is>
-          <t>wall_art</t>
+          <t>round_wall_lamp</t>
         </is>
       </c>
       <c r="F451">
@@ -51736,11 +51806,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K451" s="5" t="inlineStr">
-        <is>
-          <t>Yatak üstü + oturma alanı</t>
-        </is>
-      </c>
+      <c r="K451" s="5" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="5" t="inlineStr">
@@ -51754,7 +51820,7 @@
         </is>
       </c>
       <c r="C452" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D452">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B452)*('Kontrol Adımları'!$B$1:$B$400=C452),0),0)),"")</f>
@@ -51762,7 +51828,7 @@
       </c>
       <c r="E452" s="5" t="inlineStr">
         <is>
-          <t>cooktop</t>
+          <t>wall_art</t>
         </is>
       </c>
       <c r="F452">
@@ -51774,7 +51840,7 @@
         <v/>
       </c>
       <c r="H452" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I452" s="7" t="inlineStr">
         <is>
@@ -51786,7 +51852,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K452" s="5" t="n"/>
+      <c r="K452" s="5" t="inlineStr">
+        <is>
+          <t>Yatak üstü + oturma alanı</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="5" t="inlineStr">
@@ -51808,7 +51878,7 @@
       </c>
       <c r="E453" s="5" t="inlineStr">
         <is>
-          <t>hanging_bin</t>
+          <t>cooktop</t>
         </is>
       </c>
       <c r="F453">
@@ -51854,7 +51924,7 @@
       </c>
       <c r="E454" s="5" t="inlineStr">
         <is>
-          <t>mini_fridge</t>
+          <t>hanging_bin</t>
         </is>
       </c>
       <c r="F454">
@@ -51900,7 +51970,7 @@
       </c>
       <c r="E455" s="5" t="inlineStr">
         <is>
-          <t>range_hood</t>
+          <t>mini_fridge</t>
         </is>
       </c>
       <c r="F455">
@@ -51916,7 +51986,7 @@
       </c>
       <c r="I455" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J455" s="5" t="inlineStr">
@@ -51924,11 +51994,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K455" s="5" t="inlineStr">
-        <is>
-          <t>Üst dolap altında görünüyor</t>
-        </is>
-      </c>
+      <c r="K455" s="5" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="5" t="inlineStr">
@@ -51942,7 +52008,7 @@
         </is>
       </c>
       <c r="C456" s="5" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D456">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B456)*('Kontrol Adımları'!$B$1:$B$400=C456),0),0)),"")</f>
@@ -51950,7 +52016,7 @@
       </c>
       <c r="E456" s="5" t="inlineStr">
         <is>
-          <t>kettle</t>
+          <t>range_hood</t>
         </is>
       </c>
       <c r="F456">
@@ -51966,7 +52032,7 @@
       </c>
       <c r="I456" s="7" t="inlineStr">
         <is>
-          <t>Evet</t>
+          <t>Hayır</t>
         </is>
       </c>
       <c r="J456" s="5" t="inlineStr">
@@ -51974,7 +52040,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K456" s="5" t="n"/>
+      <c r="K456" s="5" t="inlineStr">
+        <is>
+          <t>Üst dolap altında görünüyor</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="5" t="inlineStr">
@@ -51988,7 +52058,7 @@
         </is>
       </c>
       <c r="C457" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D457">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B457)*('Kontrol Adımları'!$B$1:$B$400=C457),0),0)),"")</f>
@@ -51996,7 +52066,7 @@
       </c>
       <c r="E457" s="5" t="inlineStr">
         <is>
-          <t>paper_towel</t>
+          <t>kettle</t>
         </is>
       </c>
       <c r="F457">
@@ -52012,7 +52082,7 @@
       </c>
       <c r="I457" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J457" s="5" t="inlineStr">
@@ -52020,11 +52090,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K457" s="5" t="inlineStr">
-        <is>
-          <t>X2 ile aynı varsayıldı</t>
-        </is>
-      </c>
+      <c r="K457" s="5" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="5" t="inlineStr">
@@ -52038,7 +52104,7 @@
         </is>
       </c>
       <c r="C458" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D458">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B458)*('Kontrol Adımları'!$B$1:$B$400=C458),0),0)),"")</f>
@@ -52046,7 +52112,7 @@
       </c>
       <c r="E458" s="5" t="inlineStr">
         <is>
-          <t>air_conditioner</t>
+          <t>paper_towel</t>
         </is>
       </c>
       <c r="F458">
@@ -52062,7 +52128,7 @@
       </c>
       <c r="I458" s="7" t="inlineStr">
         <is>
-          <t>Evet</t>
+          <t>Hayır</t>
         </is>
       </c>
       <c r="J458" s="5" t="inlineStr">
@@ -52072,7 +52138,7 @@
       </c>
       <c r="K458" s="5" t="inlineStr">
         <is>
-          <t>Oturma bölümünde, banyo kapısının üstünde (video)</t>
+          <t>X2 ile aynı varsayıldı</t>
         </is>
       </c>
     </row>
@@ -52096,7 +52162,7 @@
       </c>
       <c r="E459" s="5" t="inlineStr">
         <is>
-          <t>room_bin</t>
+          <t>air_conditioner</t>
         </is>
       </c>
       <c r="F459">
@@ -52122,7 +52188,7 @@
       </c>
       <c r="K459" s="5" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Oturma bölümünde, banyo kapısının üstünde (video)</t>
         </is>
       </c>
     </row>
@@ -52134,11 +52200,11 @@
       </c>
       <c r="B460" s="5" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="C460" s="5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D460">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B460)*('Kontrol Adımları'!$B$1:$B$400=C460),0),0)),"")</f>
@@ -52146,7 +52212,7 @@
       </c>
       <c r="E460" s="5" t="inlineStr">
         <is>
-          <t>desk_with_chair</t>
+          <t>room_bin</t>
         </is>
       </c>
       <c r="F460">
@@ -52170,7 +52236,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K460" s="5" t="n"/>
+      <c r="K460" s="5" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="5" t="inlineStr">
@@ -52180,11 +52250,11 @@
       </c>
       <c r="B461" s="5" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="C461" s="5" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D461">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B461)*('Kontrol Adımları'!$B$1:$B$400=C461),0),0)),"")</f>
@@ -52192,7 +52262,7 @@
       </c>
       <c r="E461" s="5" t="inlineStr">
         <is>
-          <t>vessel_sink</t>
+          <t>ceiling_light</t>
         </is>
       </c>
       <c r="F461">
@@ -52216,7 +52286,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K461" s="5" t="n"/>
+      <c r="K461" s="5" t="inlineStr">
+        <is>
+          <t>Oturma bölümü, klima yanı (video)</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="5" t="inlineStr">
@@ -52230,7 +52304,7 @@
         </is>
       </c>
       <c r="C462" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D462">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B462)*('Kontrol Adımları'!$B$1:$B$400=C462),0),0)),"")</f>
@@ -52238,7 +52312,7 @@
       </c>
       <c r="E462" s="5" t="inlineStr">
         <is>
-          <t>basin_faucet</t>
+          <t>desk_with_chair</t>
         </is>
       </c>
       <c r="F462">
@@ -52284,7 +52358,7 @@
       </c>
       <c r="E463" s="5" t="inlineStr">
         <is>
-          <t>led_mirror</t>
+          <t>vessel_sink</t>
         </is>
       </c>
       <c r="F463">
@@ -52330,7 +52404,7 @@
       </c>
       <c r="E464" s="5" t="inlineStr">
         <is>
-          <t>liquid_soap</t>
+          <t>basin_faucet</t>
         </is>
       </c>
       <c r="F464">
@@ -52376,7 +52450,7 @@
       </c>
       <c r="E465" s="5" t="inlineStr">
         <is>
-          <t>towel_bar</t>
+          <t>led_mirror</t>
         </is>
       </c>
       <c r="F465">
@@ -52414,7 +52488,7 @@
         </is>
       </c>
       <c r="C466" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D466">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B466)*('Kontrol Adımları'!$B$1:$B$400=C466),0),0)),"")</f>
@@ -52422,7 +52496,7 @@
       </c>
       <c r="E466" s="5" t="inlineStr">
         <is>
-          <t>bath_towel</t>
+          <t>liquid_soap</t>
         </is>
       </c>
       <c r="F466">
@@ -52434,7 +52508,7 @@
         <v/>
       </c>
       <c r="H466" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I466" s="7" t="inlineStr">
         <is>
@@ -52460,7 +52534,7 @@
         </is>
       </c>
       <c r="C467" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D467">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B467)*('Kontrol Adımları'!$B$1:$B$400=C467),0),0)),"")</f>
@@ -52468,7 +52542,7 @@
       </c>
       <c r="E467" s="5" t="inlineStr">
         <is>
-          <t>hand_towel</t>
+          <t>towel_bar</t>
         </is>
       </c>
       <c r="F467">
@@ -52480,7 +52554,7 @@
         <v/>
       </c>
       <c r="H467" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I467" s="7" t="inlineStr">
         <is>
@@ -52514,7 +52588,7 @@
       </c>
       <c r="E468" s="5" t="inlineStr">
         <is>
-          <t>slippers</t>
+          <t>bath_towel</t>
         </is>
       </c>
       <c r="F468">
@@ -52560,7 +52634,7 @@
       </c>
       <c r="E469" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_spare</t>
+          <t>hand_towel</t>
         </is>
       </c>
       <c r="F469">
@@ -52572,7 +52646,7 @@
         <v/>
       </c>
       <c r="H469" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I469" s="7" t="inlineStr">
         <is>
@@ -52606,7 +52680,7 @@
       </c>
       <c r="E470" s="5" t="inlineStr">
         <is>
-          <t>hair_dryer</t>
+          <t>slippers</t>
         </is>
       </c>
       <c r="F470">
@@ -52618,7 +52692,7 @@
         <v/>
       </c>
       <c r="H470" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I470" s="7" t="inlineStr">
         <is>
@@ -52652,7 +52726,7 @@
       </c>
       <c r="E471" s="5" t="inlineStr">
         <is>
-          <t>vanity_unit</t>
+          <t>toilet_paper_spare</t>
         </is>
       </c>
       <c r="F471">
@@ -52690,7 +52764,7 @@
         </is>
       </c>
       <c r="C472" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D472">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B472)*('Kontrol Adımları'!$B$1:$B$400=C472),0),0)),"")</f>
@@ -52698,7 +52772,7 @@
       </c>
       <c r="E472" s="5" t="inlineStr">
         <is>
-          <t>wc</t>
+          <t>hair_dryer</t>
         </is>
       </c>
       <c r="F472">
@@ -52736,7 +52810,7 @@
         </is>
       </c>
       <c r="C473" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D473">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B473)*('Kontrol Adımları'!$B$1:$B$400=C473),0),0)),"")</f>
@@ -52744,7 +52818,7 @@
       </c>
       <c r="E473" s="5" t="inlineStr">
         <is>
-          <t>flush_plate</t>
+          <t>vanity_unit</t>
         </is>
       </c>
       <c r="F473">
@@ -52790,7 +52864,7 @@
       </c>
       <c r="E474" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper</t>
+          <t>wc</t>
         </is>
       </c>
       <c r="F474">
@@ -52836,7 +52910,7 @@
       </c>
       <c r="E475" s="5" t="inlineStr">
         <is>
-          <t>toilet_paper_holder</t>
+          <t>flush_plate</t>
         </is>
       </c>
       <c r="F475">
@@ -52882,7 +52956,7 @@
       </c>
       <c r="E476" s="5" t="inlineStr">
         <is>
-          <t>toilet_brush</t>
+          <t>toilet_paper</t>
         </is>
       </c>
       <c r="F476">
@@ -52928,7 +53002,7 @@
       </c>
       <c r="E477" s="5" t="inlineStr">
         <is>
-          <t>bath_bin</t>
+          <t>toilet_paper_holder</t>
         </is>
       </c>
       <c r="F477">
@@ -52966,7 +53040,7 @@
         </is>
       </c>
       <c r="C478" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D478">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B478)*('Kontrol Adımları'!$B$1:$B$400=C478),0),0)),"")</f>
@@ -52974,7 +53048,7 @@
       </c>
       <c r="E478" s="5" t="inlineStr">
         <is>
-          <t>shower_set</t>
+          <t>toilet_brush</t>
         </is>
       </c>
       <c r="F478">
@@ -53012,7 +53086,7 @@
         </is>
       </c>
       <c r="C479" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D479">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B479)*('Kontrol Adımları'!$B$1:$B$400=C479),0),0)),"")</f>
@@ -53020,7 +53094,7 @@
       </c>
       <c r="E479" s="5" t="inlineStr">
         <is>
-          <t>dispenser</t>
+          <t>bath_bin</t>
         </is>
       </c>
       <c r="F479">
@@ -53032,7 +53106,7 @@
         <v/>
       </c>
       <c r="H479" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I479" s="7" t="inlineStr">
         <is>
@@ -53066,7 +53140,7 @@
       </c>
       <c r="E480" s="5" t="inlineStr">
         <is>
-          <t>shower_basket</t>
+          <t>shower_set</t>
         </is>
       </c>
       <c r="F480">
@@ -53104,7 +53178,7 @@
         </is>
       </c>
       <c r="C481" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D481">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B481)*('Kontrol Adımları'!$B$1:$B$400=C481),0),0)),"")</f>
@@ -53112,7 +53186,7 @@
       </c>
       <c r="E481" s="5" t="inlineStr">
         <is>
-          <t>bed</t>
+          <t>dispenser</t>
         </is>
       </c>
       <c r="F481">
@@ -53124,7 +53198,7 @@
         <v/>
       </c>
       <c r="H481" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I481" s="7" t="inlineStr">
         <is>
@@ -53150,7 +53224,7 @@
         </is>
       </c>
       <c r="C482" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D482">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B482)*('Kontrol Adımları'!$B$1:$B$400=C482),0),0)),"")</f>
@@ -53158,7 +53232,7 @@
       </c>
       <c r="E482" s="5" t="inlineStr">
         <is>
-          <t>pillow</t>
+          <t>shower_basket</t>
         </is>
       </c>
       <c r="F482">
@@ -53170,7 +53244,7 @@
         <v/>
       </c>
       <c r="H482" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I482" s="7" t="inlineStr">
         <is>
@@ -53196,7 +53270,7 @@
         </is>
       </c>
       <c r="C483" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D483">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B483)*('Kontrol Adımları'!$B$1:$B$400=C483),0),0)),"")</f>
@@ -53204,7 +53278,7 @@
       </c>
       <c r="E483" s="5" t="inlineStr">
         <is>
-          <t>nightstand</t>
+          <t>bed</t>
         </is>
       </c>
       <c r="F483">
@@ -53216,7 +53290,7 @@
         <v/>
       </c>
       <c r="H483" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I483" s="7" t="inlineStr">
         <is>
@@ -53242,7 +53316,7 @@
         </is>
       </c>
       <c r="C484" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D484">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B484)*('Kontrol Adımları'!$B$1:$B$400=C484),0),0)),"")</f>
@@ -53250,7 +53324,7 @@
       </c>
       <c r="E484" s="5" t="inlineStr">
         <is>
-          <t>bedside_wall_lamp</t>
+          <t>pillow</t>
         </is>
       </c>
       <c r="F484">
@@ -53262,7 +53336,7 @@
         <v/>
       </c>
       <c r="H484" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I484" s="7" t="inlineStr">
         <is>
@@ -53288,7 +53362,7 @@
         </is>
       </c>
       <c r="C485" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D485">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B485)*('Kontrol Adımları'!$B$1:$B$400=C485),0),0)),"")</f>
@@ -53296,7 +53370,7 @@
       </c>
       <c r="E485" s="5" t="inlineStr">
         <is>
-          <t>wardrobe</t>
+          <t>nightstand</t>
         </is>
       </c>
       <c r="F485">
@@ -53308,7 +53382,7 @@
         <v/>
       </c>
       <c r="H485" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I485" s="7" t="inlineStr">
         <is>
@@ -53334,7 +53408,7 @@
         </is>
       </c>
       <c r="C486" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D486">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B486)*('Kontrol Adımları'!$B$1:$B$400=C486),0),0)),"")</f>
@@ -53342,7 +53416,7 @@
       </c>
       <c r="E486" s="5" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>bedside_wall_lamp</t>
         </is>
       </c>
       <c r="F486">
@@ -53354,11 +53428,11 @@
         <v/>
       </c>
       <c r="H486" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I486" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J486" s="5" t="inlineStr">
@@ -53366,11 +53440,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K486" s="5" t="inlineStr">
-        <is>
-          <t>Askılar sola toplanmış; fotoğrafta 4-5 görünüyor</t>
-        </is>
-      </c>
+      <c r="K486" s="5" t="n"/>
     </row>
     <row r="487" ht="39.6" customHeight="1">
       <c r="A487" s="5" t="inlineStr">
@@ -53392,7 +53462,7 @@
       </c>
       <c r="E487" s="5" t="inlineStr">
         <is>
-          <t>spare_blanket</t>
+          <t>wardrobe</t>
         </is>
       </c>
       <c r="F487">
@@ -53430,7 +53500,7 @@
         </is>
       </c>
       <c r="C488" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D488">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B488)*('Kontrol Adımları'!$B$1:$B$400=C488),0),0)),"")</f>
@@ -53438,7 +53508,7 @@
       </c>
       <c r="E488" s="5" t="inlineStr">
         <is>
-          <t>amenity_tray</t>
+          <t>hanger</t>
         </is>
       </c>
       <c r="F488">
@@ -53450,11 +53520,11 @@
         <v/>
       </c>
       <c r="H488" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I488" s="7" t="inlineStr">
         <is>
-          <t>Evet</t>
+          <t>Hayır</t>
         </is>
       </c>
       <c r="J488" s="5" t="inlineStr">
@@ -53462,7 +53532,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K488" s="5" t="n"/>
+      <c r="K488" s="5" t="inlineStr">
+        <is>
+          <t>Askılar sola toplanmış; fotoğrafta 4-5 görünüyor</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" s="5" t="inlineStr">
@@ -53476,7 +53550,7 @@
         </is>
       </c>
       <c r="C489" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D489">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B489)*('Kontrol Adımları'!$B$1:$B$400=C489),0),0)),"")</f>
@@ -53484,7 +53558,7 @@
       </c>
       <c r="E489" s="5" t="inlineStr">
         <is>
-          <t>remote</t>
+          <t>spare_blanket</t>
         </is>
       </c>
       <c r="F489">
@@ -53496,7 +53570,7 @@
         <v/>
       </c>
       <c r="H489" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I489" s="7" t="inlineStr">
         <is>
@@ -53522,7 +53596,7 @@
         </is>
       </c>
       <c r="C490" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D490">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B490)*('Kontrol Adımları'!$B$1:$B$400=C490),0),0)),"")</f>
@@ -53530,7 +53604,7 @@
       </c>
       <c r="E490" s="5" t="inlineStr">
         <is>
-          <t>sofa_gray</t>
+          <t>amenity_tray</t>
         </is>
       </c>
       <c r="F490">
@@ -53568,7 +53642,7 @@
         </is>
       </c>
       <c r="C491" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D491">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B491)*('Kontrol Adımları'!$B$1:$B$400=C491),0),0)),"")</f>
@@ -53576,7 +53650,7 @@
       </c>
       <c r="E491" s="5" t="inlineStr">
         <is>
-          <t>coffee_table_glass</t>
+          <t>remote</t>
         </is>
       </c>
       <c r="F491">
@@ -53588,7 +53662,7 @@
         <v/>
       </c>
       <c r="H491" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I491" s="7" t="inlineStr">
         <is>
@@ -53622,7 +53696,7 @@
       </c>
       <c r="E492" s="5" t="inlineStr">
         <is>
-          <t>rug_striped</t>
+          <t>sofa_gray</t>
         </is>
       </c>
       <c r="F492">
@@ -53668,7 +53742,7 @@
       </c>
       <c r="E493" s="5" t="inlineStr">
         <is>
-          <t>round_wall_lamp</t>
+          <t>coffee_table_glass</t>
         </is>
       </c>
       <c r="F493">
@@ -53680,7 +53754,7 @@
         <v/>
       </c>
       <c r="H493" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I493" s="7" t="inlineStr">
         <is>
@@ -53714,7 +53788,7 @@
       </c>
       <c r="E494" s="5" t="inlineStr">
         <is>
-          <t>decor_branches</t>
+          <t>rug_striped</t>
         </is>
       </c>
       <c r="F494">
@@ -53760,7 +53834,7 @@
       </c>
       <c r="E495" s="5" t="inlineStr">
         <is>
-          <t>wall_art</t>
+          <t>round_wall_lamp</t>
         </is>
       </c>
       <c r="F495">
@@ -53772,11 +53846,11 @@
         <v/>
       </c>
       <c r="H495" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I495" s="7" t="inlineStr">
         <is>
-          <t>Evet</t>
+          <t>Hayır</t>
         </is>
       </c>
       <c r="J495" s="5" t="inlineStr">
@@ -53786,7 +53860,7 @@
       </c>
       <c r="K495" s="5" t="inlineStr">
         <is>
-          <t>Yatak üstünde</t>
+          <t>2 kuzey duvarı (kanepe), 2 doğu duvarı (yemek ve TV yanı); teyit et</t>
         </is>
       </c>
     </row>
@@ -53802,7 +53876,7 @@
         </is>
       </c>
       <c r="C496" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D496">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B496)*('Kontrol Adımları'!$B$1:$B$400=C496),0),0)),"")</f>
@@ -53810,7 +53884,7 @@
       </c>
       <c r="E496" s="5" t="inlineStr">
         <is>
-          <t>round_table</t>
+          <t>decor_branches</t>
         </is>
       </c>
       <c r="F496">
@@ -53848,7 +53922,7 @@
         </is>
       </c>
       <c r="C497" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D497">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B497)*('Kontrol Adımları'!$B$1:$B$400=C497),0),0)),"")</f>
@@ -53856,7 +53930,7 @@
       </c>
       <c r="E497" s="5" t="inlineStr">
         <is>
-          <t>armchair</t>
+          <t>wall_art</t>
         </is>
       </c>
       <c r="F497">
@@ -53868,7 +53942,7 @@
         <v/>
       </c>
       <c r="H497" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I497" s="7" t="inlineStr">
         <is>
@@ -53880,7 +53954,11 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K497" s="5" t="n"/>
+      <c r="K497" s="5" t="inlineStr">
+        <is>
+          <t>Yatak üstünde</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" s="5" t="inlineStr">
@@ -53902,7 +53980,7 @@
       </c>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>floor_lamp</t>
+          <t>round_table</t>
         </is>
       </c>
       <c r="F498">
@@ -53948,7 +54026,7 @@
       </c>
       <c r="E499" s="5" t="inlineStr">
         <is>
-          <t>tv</t>
+          <t>armchair</t>
         </is>
       </c>
       <c r="F499">
@@ -53960,7 +54038,7 @@
         <v/>
       </c>
       <c r="H499" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I499" s="7" t="inlineStr">
         <is>
@@ -53986,7 +54064,7 @@
         </is>
       </c>
       <c r="C500" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D500">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B500)*('Kontrol Adımları'!$B$1:$B$400=C500),0),0)),"")</f>
@@ -53994,7 +54072,7 @@
       </c>
       <c r="E500" s="5" t="inlineStr">
         <is>
-          <t>cooktop</t>
+          <t>floor_lamp</t>
         </is>
       </c>
       <c r="F500">
@@ -54032,7 +54110,7 @@
         </is>
       </c>
       <c r="C501" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D501">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B501)*('Kontrol Adımları'!$B$1:$B$400=C501),0),0)),"")</f>
@@ -54040,7 +54118,7 @@
       </c>
       <c r="E501" s="5" t="inlineStr">
         <is>
-          <t>hanging_bin</t>
+          <t>tv</t>
         </is>
       </c>
       <c r="F501">
@@ -54086,7 +54164,7 @@
       </c>
       <c r="E502" s="5" t="inlineStr">
         <is>
-          <t>mini_fridge</t>
+          <t>cooktop</t>
         </is>
       </c>
       <c r="F502">
@@ -54132,7 +54210,7 @@
       </c>
       <c r="E503" s="5" t="inlineStr">
         <is>
-          <t>range_hood</t>
+          <t>hanging_bin</t>
         </is>
       </c>
       <c r="F503">
@@ -54178,7 +54256,7 @@
       </c>
       <c r="E504" s="5" t="inlineStr">
         <is>
-          <t>kettle</t>
+          <t>mini_fridge</t>
         </is>
       </c>
       <c r="F504">
@@ -54216,7 +54294,7 @@
         </is>
       </c>
       <c r="C505" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D505">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B505)*('Kontrol Adımları'!$B$1:$B$400=C505),0),0)),"")</f>
@@ -54224,7 +54302,7 @@
       </c>
       <c r="E505" s="5" t="inlineStr">
         <is>
-          <t>paper_towel</t>
+          <t>range_hood</t>
         </is>
       </c>
       <c r="F505">
@@ -54262,7 +54340,7 @@
         </is>
       </c>
       <c r="C506" s="5" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D506">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B506)*('Kontrol Adımları'!$B$1:$B$400=C506),0),0)),"")</f>
@@ -54270,7 +54348,7 @@
       </c>
       <c r="E506" s="5" t="inlineStr">
         <is>
-          <t>air_conditioner</t>
+          <t>kettle</t>
         </is>
       </c>
       <c r="F506">
@@ -54286,7 +54364,7 @@
       </c>
       <c r="I506" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J506" s="5" t="inlineStr">
@@ -54294,11 +54372,7 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K506" s="5" t="inlineStr">
-        <is>
-          <t>Fotoğraflarda görünmüyor</t>
-        </is>
-      </c>
+      <c r="K506" s="5" t="n"/>
     </row>
     <row r="507">
       <c r="A507" s="5" t="inlineStr">
@@ -54312,7 +54386,7 @@
         </is>
       </c>
       <c r="C507" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D507">
         <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B507)*('Kontrol Adımları'!$B$1:$B$400=C507),0),0)),"")</f>
@@ -54320,7 +54394,7 @@
       </c>
       <c r="E507" s="5" t="inlineStr">
         <is>
-          <t>room_bin</t>
+          <t>paper_towel</t>
         </is>
       </c>
       <c r="F507">
@@ -54336,7 +54410,7 @@
       </c>
       <c r="I507" s="7" t="inlineStr">
         <is>
-          <t>Hayır</t>
+          <t>Evet</t>
         </is>
       </c>
       <c r="J507" s="5" t="inlineStr">
@@ -54344,11 +54418,153 @@
           <t>Drive foto (20.10.2026)</t>
         </is>
       </c>
-      <c r="K507" s="5" t="inlineStr">
+      <c r="K507" s="5" t="n"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B508" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C508" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D508">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B508)*('Kontrol Adımları'!$B$1:$B$400=C508),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E508" s="5" t="inlineStr">
+        <is>
+          <t>air_conditioner</t>
+        </is>
+      </c>
+      <c r="F508">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A508)*('Kalem Kataloğu'!$B$1:$B$1000=E508),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G508">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A508)*('Kalem Kataloğu'!$B$1:$B$1000=E508),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H508" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I508" s="7" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J508" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K508" s="5" t="inlineStr">
+        <is>
+          <t>Fotoğraflarda görünmüyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B509" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C509" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D509">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B509)*('Kontrol Adımları'!$B$1:$B$400=C509),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E509" s="5" t="inlineStr">
+        <is>
+          <t>room_bin</t>
+        </is>
+      </c>
+      <c r="F509">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A509)*('Kalem Kataloğu'!$B$1:$B$1000=E509),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G509">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A509)*('Kalem Kataloğu'!$B$1:$B$1000=E509),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H509" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I509" s="7" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J509" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K509" s="5" t="inlineStr">
         <is>
           <t>Kanepe yanında siyah kova görünüyor</t>
         </is>
       </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="5" t="inlineStr">
+        <is>
+          <t>Tare Houses Hotel</t>
+        </is>
+      </c>
+      <c r="B510" s="5" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C510" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D510">
+        <f>IFERROR(INDEX('Kontrol Adımları'!$D:$D,MATCH(1,INDEX(('Kontrol Adımları'!$A$1:$A$400=B510)*('Kontrol Adımları'!$B$1:$B$400=C510),0),0)),"")</f>
+        <v/>
+      </c>
+      <c r="E510" s="5" t="inlineStr">
+        <is>
+          <t>smoke_detector</t>
+        </is>
+      </c>
+      <c r="F510">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$C$1:$C$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A510)*('Kalem Kataloğu'!$B$1:$B$1000=E510),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="G510">
+        <f>IFERROR(INDEX('Kalem Kataloğu'!$D$1:$D$1000,MATCH(1,INDEX(('Kalem Kataloğu'!$A$1:$A$1000=A510)*('Kalem Kataloğu'!$B$1:$B$1000=E510),0),0)),"?")</f>
+        <v/>
+      </c>
+      <c r="H510" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I510" s="7" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="J510" s="5" t="inlineStr">
+        <is>
+          <t>Drive foto (20.10.2026)</t>
+        </is>
+      </c>
+      <c r="K510" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K493"/>

</xml_diff>